<commit_message>
Excel: read the vector options and Value Type columns
</commit_message>
<xml_diff>
--- a/datacontract/templates/excel/odcs-template.xlsx
+++ b/datacontract/templates/excel/odcs-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jakob/entropyData/open-data-contract-standard-excel-template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{342FE4F4-9DE3-3540-BE91-7790BCC57F23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB75899B-EBE7-F043-8A3F-9BE4C8EF552B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="-33240" windowWidth="60160" windowHeight="33240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="8" r:id="rId1"/>
@@ -40,7 +40,7 @@
     <definedName name="authoritativeDefinitions">'Authoritative Definitions'!$A$4:$F$1000</definedName>
     <definedName name="constraints">Constraints!$A$4:$AZ$1000</definedName>
     <definedName name="context.instructions">Fundamentals!$C$25</definedName>
-    <definedName name="CustomProperties">'Custom Properties'!$A$5:$G$21</definedName>
+    <definedName name="CustomProperties">'Custom Properties'!$A$5:$H$21</definedName>
     <definedName name="datacontract_id">Fundamentals!$C$7</definedName>
     <definedName name="dataProduct">Fundamentals!$C$15</definedName>
     <definedName name="description.limitations">Fundamentals!$C$20</definedName>
@@ -69,7 +69,7 @@
     <definedName name="schema.name" localSheetId="2">'Schema &lt;table_name&gt;'!$B$5</definedName>
     <definedName name="schema.physicalName" localSheetId="2">'Schema &lt;table_name&gt;'!$B$9</definedName>
     <definedName name="schema.physicalType" localSheetId="2">'Schema &lt;table_name&gt;'!$B$6</definedName>
-    <definedName name="schema.properties" localSheetId="2">'Schema &lt;table_name&gt;'!$A$16:$AO$984</definedName>
+    <definedName name="schema.properties" localSheetId="2">'Schema &lt;table_name&gt;'!$A$16:$AU$984</definedName>
     <definedName name="schema.tags" localSheetId="2">'Schema &lt;table_name&gt;'!$B$11</definedName>
     <definedName name="servers.account">Servers!$C$11</definedName>
     <definedName name="servers.catalog">Servers!$C$12</definedName>
@@ -132,7 +132,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="257">
   <si>
     <t>Property</t>
   </si>
@@ -905,6 +905,30 @@
   <si>
     <t xml:space="preserve">This section lists the roles that a consumer may need to access the dataset depending on the type of access they require.
 </t>
+  </si>
+  <si>
+    <t>Dimensions</t>
+  </si>
+  <si>
+    <t>Element Type</t>
+  </si>
+  <si>
+    <t>Distance Metric</t>
+  </si>
+  <si>
+    <t>Normalized</t>
+  </si>
+  <si>
+    <t>Embedding Model</t>
+  </si>
+  <si>
+    <t>Embedding Model Version</t>
+  </si>
+  <si>
+    <t>Value Type</t>
+  </si>
+  <si>
+    <t>Text</t>
   </si>
 </sst>
 </file>
@@ -14328,35 +14352,36 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29635FC6-19E5-6E43-84D3-3161FAC792B3}">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.6640625" style="2" customWidth="1"/>
     <col min="2" max="2" width="22.5" style="2" customWidth="1"/>
     <col min="3" max="3" width="33.1640625" style="2" customWidth="1"/>
     <col min="4" max="4" width="43.1640625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="36.6640625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="28.5" style="2" customWidth="1"/>
-    <col min="7" max="7" width="30" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="8.83203125" style="2"/>
+    <col min="5" max="5" width="11.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="36.6640625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="28.5" style="2" customWidth="1"/>
+    <col min="8" max="8" width="30" style="2" customWidth="1"/>
+    <col min="9" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="24" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="9" t="s">
         <v>55</v>
       </c>
@@ -14370,16 +14395,19 @@
         <v>1</v>
       </c>
       <c r="E4" s="10" t="s">
+        <v>255</v>
+      </c>
+      <c r="F4" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="G4" s="10" t="s">
         <v>216</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="H4" s="10" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5" t="s">
@@ -14389,159 +14417,213 @@
         <f>IF(owner &lt;&gt; "", owner, "")</f>
         <v/>
       </c>
-      <c r="E5" s="5"/>
+      <c r="E5" s="5" t="s">
+        <v>256</v>
+      </c>
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H5" s="5"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
+      <c r="E6" s="5" t="s">
+        <v>256</v>
+      </c>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H6" s="5"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
+      <c r="E7" s="5" t="s">
+        <v>256</v>
+      </c>
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H7" s="5"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
+      <c r="E8" s="5" t="s">
+        <v>256</v>
+      </c>
       <c r="F8" s="5"/>
       <c r="G8" s="5"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H8" s="5"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
+      <c r="E9" s="5" t="s">
+        <v>256</v>
+      </c>
       <c r="F9" s="5"/>
       <c r="G9" s="5"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H9" s="5"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
+      <c r="E10" s="5" t="s">
+        <v>256</v>
+      </c>
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H10" s="5"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
+      <c r="E11" s="5" t="s">
+        <v>256</v>
+      </c>
       <c r="F11" s="5"/>
       <c r="G11" s="5"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H11" s="5"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
+      <c r="E12" s="5" t="s">
+        <v>256</v>
+      </c>
       <c r="F12" s="5"/>
       <c r="G12" s="5"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H12" s="5"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
+      <c r="E13" s="5" t="s">
+        <v>256</v>
+      </c>
       <c r="F13" s="5"/>
       <c r="G13" s="5"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H13" s="5"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
+      <c r="E14" s="5" t="s">
+        <v>256</v>
+      </c>
       <c r="F14" s="5"/>
       <c r="G14" s="5"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H14" s="5"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
+      <c r="E15" s="5" t="s">
+        <v>256</v>
+      </c>
       <c r="F15" s="5"/>
       <c r="G15" s="5"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H15" s="5"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
+      <c r="E16" s="5" t="s">
+        <v>256</v>
+      </c>
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H16" s="5"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
+      <c r="E17" s="5" t="s">
+        <v>256</v>
+      </c>
       <c r="F17" s="5"/>
       <c r="G17" s="5"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H17" s="5"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
       <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
+      <c r="E18" s="5" t="s">
+        <v>256</v>
+      </c>
       <c r="F18" s="5"/>
       <c r="G18" s="5"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H18" s="5"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="5"/>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
+      <c r="E19" s="5" t="s">
+        <v>256</v>
+      </c>
       <c r="F19" s="5"/>
       <c r="G19" s="5"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H19" s="5"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
       <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
+      <c r="E20" s="5" t="s">
+        <v>256</v>
+      </c>
       <c r="F20" s="5"/>
       <c r="G20" s="5"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H20" s="5"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="5"/>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
       <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
+      <c r="E21" s="5" t="s">
+        <v>256</v>
+      </c>
       <c r="F21" s="5"/>
       <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation allowBlank="1" sqref="D5:D61 E5:G21 B5:B22" xr:uid="{39D00745-E29F-BB4D-8EFF-9275524C1814}"/>
+  <dataValidations count="3">
+    <dataValidation allowBlank="1" sqref="B5:B22 F5:H21 D5:D61" xr:uid="{39D00745-E29F-BB4D-8EFF-9275524C1814}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A5:A100" xr:uid="{9046F39E-9EB3-EF47-83AF-F83388AB159D}">
       <formula1>"Contract,Description,Server,Schema,Property,Enum Value,Synonym,Relationship,Quality,Support,Team,Team Member,Role,SLA,Verified Statement,Constraint"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="E5:E100" xr:uid="{FD2B148B-B740-B14F-B337-F0CE13B025AB}">
+      <formula1>"Text,JSON"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15500,7 +15582,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AR52"/>
+  <dimension ref="A1:AX52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.83203125" style="2" customWidth="1"/>
@@ -15521,28 +15603,28 @@
     <col min="18" max="22" width="19" style="2" customWidth="1"/>
     <col min="23" max="23" width="21.6640625" style="2" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="27.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="25" max="40" width="15.5" style="2" customWidth="1"/>
-    <col min="41" max="41" width="44.33203125" style="2" customWidth="1"/>
-    <col min="42" max="44" width="15.83203125" style="2" customWidth="1"/>
-    <col min="45" max="16384" width="8.83203125" style="2"/>
+    <col min="25" max="46" width="15.5" style="2" customWidth="1"/>
+    <col min="47" max="47" width="44.33203125" style="2" customWidth="1"/>
+    <col min="48" max="50" width="15.83203125" style="2" customWidth="1"/>
+    <col min="51" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:44" ht="24" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:50" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="5" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
         <v>8</v>
       </c>
@@ -15553,7 +15635,7 @@
       <c r="D5" s="36"/>
       <c r="E5" s="36"/>
     </row>
-    <row r="6" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
         <v>18</v>
       </c>
@@ -15564,7 +15646,7 @@
       <c r="D6" s="36"/>
       <c r="E6" s="36"/>
     </row>
-    <row r="7" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
         <v>3</v>
       </c>
@@ -15573,7 +15655,7 @@
       <c r="D7" s="36"/>
       <c r="E7" s="36"/>
     </row>
-    <row r="8" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
         <v>9</v>
       </c>
@@ -15582,7 +15664,7 @@
       <c r="D8" s="38"/>
       <c r="E8" s="39"/>
     </row>
-    <row r="9" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
         <v>51</v>
       </c>
@@ -15591,7 +15673,7 @@
       <c r="D9" s="38"/>
       <c r="E9" s="39"/>
     </row>
-    <row r="10" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
         <v>52</v>
       </c>
@@ -15600,7 +15682,7 @@
       <c r="D10" s="38"/>
       <c r="E10" s="39"/>
     </row>
-    <row r="11" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
         <v>12</v>
       </c>
@@ -15609,7 +15691,7 @@
       <c r="D11" s="36"/>
       <c r="E11" s="36"/>
     </row>
-    <row r="12" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
         <v>22</v>
       </c>
@@ -15618,7 +15700,7 @@
       <c r="D12" s="36"/>
       <c r="E12" s="36"/>
     </row>
-    <row r="13" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
         <v>242</v>
       </c>
@@ -15627,7 +15709,7 @@
       <c r="D13" s="36"/>
       <c r="E13" s="36"/>
     </row>
-    <row r="14" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
         <v>218</v>
       </c>
@@ -15636,7 +15718,7 @@
       <c r="D14" s="36"/>
       <c r="E14" s="36"/>
     </row>
-    <row r="15" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:50" x14ac:dyDescent="0.2">
       <c r="E15" s="2"/>
       <c r="Y15" s="19" t="s">
         <v>77</v>
@@ -15654,14 +15736,20 @@
       <c r="AJ15" s="20"/>
       <c r="AK15" s="20"/>
       <c r="AL15" s="20"/>
-      <c r="AM15" s="21"/>
-      <c r="AP15" s="19" t="s">
-        <v>31</v>
-      </c>
+      <c r="AM15" s="20"/>
+      <c r="AN15" s="20"/>
+      <c r="AO15" s="20"/>
+      <c r="AP15" s="20"/>
       <c r="AQ15" s="20"/>
       <c r="AR15" s="20"/>
-    </row>
-    <row r="16" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS15" s="21"/>
+      <c r="AV15" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="AW15" s="20"/>
+      <c r="AX15" s="20"/>
+    </row>
+    <row r="16" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
         <v>0</v>
       </c>
@@ -15780,16 +15868,34 @@
         <v>87</v>
       </c>
       <c r="AN16" s="10" t="s">
+        <v>249</v>
+      </c>
+      <c r="AO16" s="10" t="s">
+        <v>250</v>
+      </c>
+      <c r="AP16" s="10" t="s">
+        <v>251</v>
+      </c>
+      <c r="AQ16" s="10" t="s">
+        <v>252</v>
+      </c>
+      <c r="AR16" s="10" t="s">
+        <v>253</v>
+      </c>
+      <c r="AS16" s="10" t="s">
+        <v>254</v>
+      </c>
+      <c r="AT16" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="AO16" s="10" t="s">
+      <c r="AU16" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="AP16" s="10"/>
-      <c r="AQ16" s="10"/>
-      <c r="AR16" s="10"/>
-    </row>
-    <row r="17" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AV16" s="10"/>
+      <c r="AW16" s="10"/>
+      <c r="AX16" s="10"/>
+    </row>
+    <row r="17" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A17" s="17"/>
       <c r="B17" s="15"/>
       <c r="C17" s="15"/>
@@ -15820,22 +15926,28 @@
       <c r="AB17" s="15"/>
       <c r="AC17" s="15"/>
       <c r="AD17" s="15"/>
-      <c r="AE17" s="15"/>
-      <c r="AF17" s="15"/>
-      <c r="AG17" s="15"/>
-      <c r="AH17" s="15"/>
+      <c r="AE17" s="16"/>
+      <c r="AF17" s="16"/>
+      <c r="AG17" s="16"/>
+      <c r="AH17" s="16"/>
       <c r="AI17" s="15"/>
       <c r="AJ17" s="15"/>
       <c r="AK17" s="15"/>
       <c r="AL17" s="15"/>
       <c r="AM17" s="15"/>
       <c r="AN17" s="15"/>
-      <c r="AO17" s="28"/>
+      <c r="AO17" s="15"/>
       <c r="AP17" s="15"/>
       <c r="AQ17" s="15"/>
       <c r="AR17" s="15"/>
-    </row>
-    <row r="18" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS17" s="15"/>
+      <c r="AT17" s="15"/>
+      <c r="AU17" s="28"/>
+      <c r="AV17" s="15"/>
+      <c r="AW17" s="15"/>
+      <c r="AX17" s="15"/>
+    </row>
+    <row r="18" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A18" s="17"/>
       <c r="B18" s="15"/>
       <c r="C18" s="15"/>
@@ -15866,22 +15978,28 @@
       <c r="AB18" s="15"/>
       <c r="AC18" s="15"/>
       <c r="AD18" s="15"/>
-      <c r="AE18" s="15"/>
-      <c r="AF18" s="15"/>
-      <c r="AG18" s="15"/>
-      <c r="AH18" s="15"/>
+      <c r="AE18" s="16"/>
+      <c r="AF18" s="16"/>
+      <c r="AG18" s="16"/>
+      <c r="AH18" s="16"/>
       <c r="AI18" s="15"/>
       <c r="AJ18" s="15"/>
       <c r="AK18" s="15"/>
       <c r="AL18" s="15"/>
       <c r="AM18" s="15"/>
       <c r="AN18" s="15"/>
-      <c r="AO18" s="28"/>
+      <c r="AO18" s="15"/>
       <c r="AP18" s="15"/>
       <c r="AQ18" s="15"/>
       <c r="AR18" s="15"/>
-    </row>
-    <row r="19" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS18" s="15"/>
+      <c r="AT18" s="15"/>
+      <c r="AU18" s="28"/>
+      <c r="AV18" s="15"/>
+      <c r="AW18" s="15"/>
+      <c r="AX18" s="15"/>
+    </row>
+    <row r="19" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A19" s="17"/>
       <c r="B19" s="15"/>
       <c r="C19" s="15"/>
@@ -15912,22 +16030,28 @@
       <c r="AB19" s="15"/>
       <c r="AC19" s="15"/>
       <c r="AD19" s="15"/>
-      <c r="AE19" s="15"/>
-      <c r="AF19" s="15"/>
-      <c r="AG19" s="15"/>
-      <c r="AH19" s="15"/>
+      <c r="AE19" s="16"/>
+      <c r="AF19" s="16"/>
+      <c r="AG19" s="16"/>
+      <c r="AH19" s="16"/>
       <c r="AI19" s="15"/>
       <c r="AJ19" s="15"/>
       <c r="AK19" s="15"/>
       <c r="AL19" s="15"/>
       <c r="AM19" s="15"/>
       <c r="AN19" s="15"/>
-      <c r="AO19" s="28"/>
+      <c r="AO19" s="15"/>
       <c r="AP19" s="15"/>
       <c r="AQ19" s="15"/>
       <c r="AR19" s="15"/>
-    </row>
-    <row r="20" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS19" s="15"/>
+      <c r="AT19" s="15"/>
+      <c r="AU19" s="28"/>
+      <c r="AV19" s="15"/>
+      <c r="AW19" s="15"/>
+      <c r="AX19" s="15"/>
+    </row>
+    <row r="20" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A20" s="17"/>
       <c r="B20" s="15"/>
       <c r="C20" s="15"/>
@@ -15958,22 +16082,28 @@
       <c r="AB20" s="15"/>
       <c r="AC20" s="15"/>
       <c r="AD20" s="15"/>
-      <c r="AE20" s="15"/>
-      <c r="AF20" s="15"/>
-      <c r="AG20" s="15"/>
-      <c r="AH20" s="15"/>
+      <c r="AE20" s="16"/>
+      <c r="AF20" s="16"/>
+      <c r="AG20" s="16"/>
+      <c r="AH20" s="16"/>
       <c r="AI20" s="15"/>
       <c r="AJ20" s="15"/>
       <c r="AK20" s="15"/>
       <c r="AL20" s="15"/>
       <c r="AM20" s="15"/>
       <c r="AN20" s="15"/>
-      <c r="AO20" s="28"/>
+      <c r="AO20" s="15"/>
       <c r="AP20" s="15"/>
       <c r="AQ20" s="15"/>
       <c r="AR20" s="15"/>
-    </row>
-    <row r="21" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS20" s="15"/>
+      <c r="AT20" s="15"/>
+      <c r="AU20" s="28"/>
+      <c r="AV20" s="15"/>
+      <c r="AW20" s="15"/>
+      <c r="AX20" s="15"/>
+    </row>
+    <row r="21" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A21" s="17"/>
       <c r="B21" s="15"/>
       <c r="C21" s="15"/>
@@ -16004,22 +16134,28 @@
       <c r="AB21" s="15"/>
       <c r="AC21" s="15"/>
       <c r="AD21" s="15"/>
-      <c r="AE21" s="15"/>
-      <c r="AF21" s="15"/>
-      <c r="AG21" s="15"/>
-      <c r="AH21" s="15"/>
+      <c r="AE21" s="16"/>
+      <c r="AF21" s="16"/>
+      <c r="AG21" s="16"/>
+      <c r="AH21" s="16"/>
       <c r="AI21" s="15"/>
       <c r="AJ21" s="15"/>
       <c r="AK21" s="15"/>
       <c r="AL21" s="15"/>
       <c r="AM21" s="15"/>
       <c r="AN21" s="15"/>
-      <c r="AO21" s="28"/>
+      <c r="AO21" s="15"/>
       <c r="AP21" s="15"/>
       <c r="AQ21" s="15"/>
       <c r="AR21" s="15"/>
-    </row>
-    <row r="22" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS21" s="15"/>
+      <c r="AT21" s="15"/>
+      <c r="AU21" s="28"/>
+      <c r="AV21" s="15"/>
+      <c r="AW21" s="15"/>
+      <c r="AX21" s="15"/>
+    </row>
+    <row r="22" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A22" s="17"/>
       <c r="B22" s="15"/>
       <c r="C22" s="15"/>
@@ -16050,22 +16186,28 @@
       <c r="AB22" s="15"/>
       <c r="AC22" s="15"/>
       <c r="AD22" s="15"/>
-      <c r="AE22" s="15"/>
-      <c r="AF22" s="15"/>
-      <c r="AG22" s="15"/>
-      <c r="AH22" s="15"/>
+      <c r="AE22" s="16"/>
+      <c r="AF22" s="16"/>
+      <c r="AG22" s="16"/>
+      <c r="AH22" s="16"/>
       <c r="AI22" s="15"/>
       <c r="AJ22" s="15"/>
       <c r="AK22" s="15"/>
       <c r="AL22" s="15"/>
       <c r="AM22" s="15"/>
       <c r="AN22" s="15"/>
-      <c r="AO22" s="28"/>
+      <c r="AO22" s="15"/>
       <c r="AP22" s="15"/>
       <c r="AQ22" s="15"/>
       <c r="AR22" s="15"/>
-    </row>
-    <row r="23" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS22" s="15"/>
+      <c r="AT22" s="15"/>
+      <c r="AU22" s="28"/>
+      <c r="AV22" s="15"/>
+      <c r="AW22" s="15"/>
+      <c r="AX22" s="15"/>
+    </row>
+    <row r="23" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A23" s="17"/>
       <c r="B23" s="15"/>
       <c r="C23" s="15"/>
@@ -16096,22 +16238,28 @@
       <c r="AB23" s="15"/>
       <c r="AC23" s="15"/>
       <c r="AD23" s="15"/>
-      <c r="AE23" s="15"/>
-      <c r="AF23" s="15"/>
-      <c r="AG23" s="15"/>
-      <c r="AH23" s="15"/>
+      <c r="AE23" s="16"/>
+      <c r="AF23" s="16"/>
+      <c r="AG23" s="16"/>
+      <c r="AH23" s="16"/>
       <c r="AI23" s="15"/>
       <c r="AJ23" s="15"/>
       <c r="AK23" s="15"/>
       <c r="AL23" s="15"/>
       <c r="AM23" s="15"/>
       <c r="AN23" s="15"/>
-      <c r="AO23" s="28"/>
+      <c r="AO23" s="15"/>
       <c r="AP23" s="15"/>
       <c r="AQ23" s="15"/>
       <c r="AR23" s="15"/>
-    </row>
-    <row r="24" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS23" s="15"/>
+      <c r="AT23" s="15"/>
+      <c r="AU23" s="28"/>
+      <c r="AV23" s="15"/>
+      <c r="AW23" s="15"/>
+      <c r="AX23" s="15"/>
+    </row>
+    <row r="24" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A24" s="18"/>
       <c r="B24" s="15"/>
       <c r="C24" s="15"/>
@@ -16142,22 +16290,28 @@
       <c r="AB24" s="15"/>
       <c r="AC24" s="15"/>
       <c r="AD24" s="15"/>
-      <c r="AE24" s="15"/>
-      <c r="AF24" s="15"/>
-      <c r="AG24" s="15"/>
-      <c r="AH24" s="15"/>
+      <c r="AE24" s="16"/>
+      <c r="AF24" s="16"/>
+      <c r="AG24" s="16"/>
+      <c r="AH24" s="16"/>
       <c r="AI24" s="15"/>
       <c r="AJ24" s="15"/>
       <c r="AK24" s="15"/>
       <c r="AL24" s="15"/>
       <c r="AM24" s="15"/>
       <c r="AN24" s="15"/>
-      <c r="AO24" s="28"/>
+      <c r="AO24" s="15"/>
       <c r="AP24" s="15"/>
       <c r="AQ24" s="15"/>
       <c r="AR24" s="15"/>
-    </row>
-    <row r="25" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS24" s="15"/>
+      <c r="AT24" s="15"/>
+      <c r="AU24" s="28"/>
+      <c r="AV24" s="15"/>
+      <c r="AW24" s="15"/>
+      <c r="AX24" s="15"/>
+    </row>
+    <row r="25" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A25" s="18"/>
       <c r="B25" s="15"/>
       <c r="C25" s="15"/>
@@ -16188,22 +16342,28 @@
       <c r="AB25" s="15"/>
       <c r="AC25" s="15"/>
       <c r="AD25" s="15"/>
-      <c r="AE25" s="15"/>
-      <c r="AF25" s="15"/>
-      <c r="AG25" s="15"/>
-      <c r="AH25" s="15"/>
+      <c r="AE25" s="16"/>
+      <c r="AF25" s="16"/>
+      <c r="AG25" s="16"/>
+      <c r="AH25" s="16"/>
       <c r="AI25" s="15"/>
       <c r="AJ25" s="15"/>
       <c r="AK25" s="15"/>
       <c r="AL25" s="15"/>
       <c r="AM25" s="15"/>
       <c r="AN25" s="15"/>
-      <c r="AO25" s="28"/>
+      <c r="AO25" s="15"/>
       <c r="AP25" s="15"/>
       <c r="AQ25" s="15"/>
       <c r="AR25" s="15"/>
-    </row>
-    <row r="26" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS25" s="15"/>
+      <c r="AT25" s="15"/>
+      <c r="AU25" s="28"/>
+      <c r="AV25" s="15"/>
+      <c r="AW25" s="15"/>
+      <c r="AX25" s="15"/>
+    </row>
+    <row r="26" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A26" s="18"/>
       <c r="B26" s="15"/>
       <c r="C26" s="15"/>
@@ -16234,22 +16394,28 @@
       <c r="AB26" s="15"/>
       <c r="AC26" s="15"/>
       <c r="AD26" s="15"/>
-      <c r="AE26" s="15"/>
-      <c r="AF26" s="15"/>
-      <c r="AG26" s="15"/>
-      <c r="AH26" s="15"/>
+      <c r="AE26" s="16"/>
+      <c r="AF26" s="16"/>
+      <c r="AG26" s="16"/>
+      <c r="AH26" s="16"/>
       <c r="AI26" s="15"/>
       <c r="AJ26" s="15"/>
       <c r="AK26" s="15"/>
       <c r="AL26" s="15"/>
       <c r="AM26" s="15"/>
       <c r="AN26" s="15"/>
-      <c r="AO26" s="28"/>
+      <c r="AO26" s="15"/>
       <c r="AP26" s="15"/>
       <c r="AQ26" s="15"/>
       <c r="AR26" s="15"/>
-    </row>
-    <row r="27" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS26" s="15"/>
+      <c r="AT26" s="15"/>
+      <c r="AU26" s="28"/>
+      <c r="AV26" s="15"/>
+      <c r="AW26" s="15"/>
+      <c r="AX26" s="15"/>
+    </row>
+    <row r="27" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A27" s="17"/>
       <c r="B27" s="15"/>
       <c r="C27" s="15"/>
@@ -16280,22 +16446,28 @@
       <c r="AB27" s="15"/>
       <c r="AC27" s="15"/>
       <c r="AD27" s="15"/>
-      <c r="AE27" s="15"/>
-      <c r="AF27" s="15"/>
-      <c r="AG27" s="15"/>
-      <c r="AH27" s="15"/>
+      <c r="AE27" s="16"/>
+      <c r="AF27" s="16"/>
+      <c r="AG27" s="16"/>
+      <c r="AH27" s="16"/>
       <c r="AI27" s="15"/>
       <c r="AJ27" s="15"/>
       <c r="AK27" s="15"/>
       <c r="AL27" s="15"/>
       <c r="AM27" s="15"/>
       <c r="AN27" s="15"/>
-      <c r="AO27" s="28"/>
+      <c r="AO27" s="15"/>
       <c r="AP27" s="15"/>
       <c r="AQ27" s="15"/>
       <c r="AR27" s="15"/>
-    </row>
-    <row r="28" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS27" s="15"/>
+      <c r="AT27" s="15"/>
+      <c r="AU27" s="28"/>
+      <c r="AV27" s="15"/>
+      <c r="AW27" s="15"/>
+      <c r="AX27" s="15"/>
+    </row>
+    <row r="28" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A28" s="17"/>
       <c r="B28" s="15"/>
       <c r="C28" s="15"/>
@@ -16326,22 +16498,28 @@
       <c r="AB28" s="15"/>
       <c r="AC28" s="15"/>
       <c r="AD28" s="15"/>
-      <c r="AE28" s="15"/>
-      <c r="AF28" s="15"/>
-      <c r="AG28" s="15"/>
-      <c r="AH28" s="15"/>
+      <c r="AE28" s="16"/>
+      <c r="AF28" s="16"/>
+      <c r="AG28" s="16"/>
+      <c r="AH28" s="16"/>
       <c r="AI28" s="15"/>
       <c r="AJ28" s="15"/>
       <c r="AK28" s="15"/>
       <c r="AL28" s="15"/>
       <c r="AM28" s="15"/>
       <c r="AN28" s="15"/>
-      <c r="AO28" s="28"/>
+      <c r="AO28" s="15"/>
       <c r="AP28" s="15"/>
       <c r="AQ28" s="15"/>
       <c r="AR28" s="15"/>
-    </row>
-    <row r="29" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS28" s="15"/>
+      <c r="AT28" s="15"/>
+      <c r="AU28" s="28"/>
+      <c r="AV28" s="15"/>
+      <c r="AW28" s="15"/>
+      <c r="AX28" s="15"/>
+    </row>
+    <row r="29" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A29" s="17"/>
       <c r="B29" s="15"/>
       <c r="C29" s="15"/>
@@ -16372,22 +16550,28 @@
       <c r="AB29" s="15"/>
       <c r="AC29" s="15"/>
       <c r="AD29" s="15"/>
-      <c r="AE29" s="15"/>
-      <c r="AF29" s="15"/>
-      <c r="AG29" s="15"/>
-      <c r="AH29" s="15"/>
+      <c r="AE29" s="16"/>
+      <c r="AF29" s="16"/>
+      <c r="AG29" s="16"/>
+      <c r="AH29" s="16"/>
       <c r="AI29" s="15"/>
       <c r="AJ29" s="15"/>
       <c r="AK29" s="15"/>
       <c r="AL29" s="15"/>
       <c r="AM29" s="15"/>
       <c r="AN29" s="15"/>
-      <c r="AO29" s="28"/>
+      <c r="AO29" s="15"/>
       <c r="AP29" s="15"/>
       <c r="AQ29" s="15"/>
       <c r="AR29" s="15"/>
-    </row>
-    <row r="30" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS29" s="15"/>
+      <c r="AT29" s="15"/>
+      <c r="AU29" s="28"/>
+      <c r="AV29" s="15"/>
+      <c r="AW29" s="15"/>
+      <c r="AX29" s="15"/>
+    </row>
+    <row r="30" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A30" s="17"/>
       <c r="B30" s="15"/>
       <c r="C30" s="15"/>
@@ -16418,22 +16602,28 @@
       <c r="AB30" s="15"/>
       <c r="AC30" s="15"/>
       <c r="AD30" s="15"/>
-      <c r="AE30" s="15"/>
-      <c r="AF30" s="15"/>
-      <c r="AG30" s="15"/>
-      <c r="AH30" s="15"/>
+      <c r="AE30" s="16"/>
+      <c r="AF30" s="16"/>
+      <c r="AG30" s="16"/>
+      <c r="AH30" s="16"/>
       <c r="AI30" s="15"/>
       <c r="AJ30" s="15"/>
       <c r="AK30" s="15"/>
       <c r="AL30" s="15"/>
       <c r="AM30" s="15"/>
       <c r="AN30" s="15"/>
-      <c r="AO30" s="28"/>
+      <c r="AO30" s="15"/>
       <c r="AP30" s="15"/>
       <c r="AQ30" s="15"/>
       <c r="AR30" s="15"/>
-    </row>
-    <row r="31" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS30" s="15"/>
+      <c r="AT30" s="15"/>
+      <c r="AU30" s="28"/>
+      <c r="AV30" s="15"/>
+      <c r="AW30" s="15"/>
+      <c r="AX30" s="15"/>
+    </row>
+    <row r="31" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A31" s="17"/>
       <c r="B31" s="15"/>
       <c r="C31" s="15"/>
@@ -16464,22 +16654,28 @@
       <c r="AB31" s="15"/>
       <c r="AC31" s="15"/>
       <c r="AD31" s="15"/>
-      <c r="AE31" s="15"/>
-      <c r="AF31" s="15"/>
-      <c r="AG31" s="15"/>
-      <c r="AH31" s="15"/>
+      <c r="AE31" s="16"/>
+      <c r="AF31" s="16"/>
+      <c r="AG31" s="16"/>
+      <c r="AH31" s="16"/>
       <c r="AI31" s="15"/>
       <c r="AJ31" s="15"/>
       <c r="AK31" s="15"/>
       <c r="AL31" s="15"/>
       <c r="AM31" s="15"/>
       <c r="AN31" s="15"/>
-      <c r="AO31" s="28"/>
+      <c r="AO31" s="15"/>
       <c r="AP31" s="15"/>
       <c r="AQ31" s="15"/>
       <c r="AR31" s="15"/>
-    </row>
-    <row r="32" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS31" s="15"/>
+      <c r="AT31" s="15"/>
+      <c r="AU31" s="28"/>
+      <c r="AV31" s="15"/>
+      <c r="AW31" s="15"/>
+      <c r="AX31" s="15"/>
+    </row>
+    <row r="32" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A32" s="17"/>
       <c r="B32" s="15"/>
       <c r="C32" s="15"/>
@@ -16510,22 +16706,28 @@
       <c r="AB32" s="15"/>
       <c r="AC32" s="15"/>
       <c r="AD32" s="15"/>
-      <c r="AE32" s="15"/>
-      <c r="AF32" s="15"/>
-      <c r="AG32" s="15"/>
-      <c r="AH32" s="15"/>
+      <c r="AE32" s="16"/>
+      <c r="AF32" s="16"/>
+      <c r="AG32" s="16"/>
+      <c r="AH32" s="16"/>
       <c r="AI32" s="15"/>
       <c r="AJ32" s="15"/>
       <c r="AK32" s="15"/>
       <c r="AL32" s="15"/>
       <c r="AM32" s="15"/>
       <c r="AN32" s="15"/>
-      <c r="AO32" s="28"/>
+      <c r="AO32" s="15"/>
       <c r="AP32" s="15"/>
       <c r="AQ32" s="15"/>
       <c r="AR32" s="15"/>
-    </row>
-    <row r="33" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS32" s="15"/>
+      <c r="AT32" s="15"/>
+      <c r="AU32" s="28"/>
+      <c r="AV32" s="15"/>
+      <c r="AW32" s="15"/>
+      <c r="AX32" s="15"/>
+    </row>
+    <row r="33" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A33" s="17"/>
       <c r="B33" s="15"/>
       <c r="C33" s="15"/>
@@ -16556,22 +16758,28 @@
       <c r="AB33" s="15"/>
       <c r="AC33" s="15"/>
       <c r="AD33" s="15"/>
-      <c r="AE33" s="15"/>
-      <c r="AF33" s="15"/>
-      <c r="AG33" s="15"/>
-      <c r="AH33" s="15"/>
+      <c r="AE33" s="16"/>
+      <c r="AF33" s="16"/>
+      <c r="AG33" s="16"/>
+      <c r="AH33" s="16"/>
       <c r="AI33" s="15"/>
       <c r="AJ33" s="15"/>
       <c r="AK33" s="15"/>
       <c r="AL33" s="15"/>
       <c r="AM33" s="15"/>
       <c r="AN33" s="15"/>
-      <c r="AO33" s="28"/>
+      <c r="AO33" s="15"/>
       <c r="AP33" s="15"/>
       <c r="AQ33" s="15"/>
       <c r="AR33" s="15"/>
-    </row>
-    <row r="34" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS33" s="15"/>
+      <c r="AT33" s="15"/>
+      <c r="AU33" s="28"/>
+      <c r="AV33" s="15"/>
+      <c r="AW33" s="15"/>
+      <c r="AX33" s="15"/>
+    </row>
+    <row r="34" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A34" s="17"/>
       <c r="B34" s="15"/>
       <c r="C34" s="15"/>
@@ -16602,22 +16810,28 @@
       <c r="AB34" s="15"/>
       <c r="AC34" s="15"/>
       <c r="AD34" s="15"/>
-      <c r="AE34" s="15"/>
-      <c r="AF34" s="15"/>
-      <c r="AG34" s="15"/>
-      <c r="AH34" s="15"/>
+      <c r="AE34" s="16"/>
+      <c r="AF34" s="16"/>
+      <c r="AG34" s="16"/>
+      <c r="AH34" s="16"/>
       <c r="AI34" s="15"/>
       <c r="AJ34" s="15"/>
       <c r="AK34" s="15"/>
       <c r="AL34" s="15"/>
       <c r="AM34" s="15"/>
       <c r="AN34" s="15"/>
-      <c r="AO34" s="28"/>
+      <c r="AO34" s="15"/>
       <c r="AP34" s="15"/>
       <c r="AQ34" s="15"/>
       <c r="AR34" s="15"/>
-    </row>
-    <row r="35" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS34" s="15"/>
+      <c r="AT34" s="15"/>
+      <c r="AU34" s="28"/>
+      <c r="AV34" s="15"/>
+      <c r="AW34" s="15"/>
+      <c r="AX34" s="15"/>
+    </row>
+    <row r="35" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A35" s="17"/>
       <c r="B35" s="15"/>
       <c r="C35" s="15"/>
@@ -16648,22 +16862,28 @@
       <c r="AB35" s="15"/>
       <c r="AC35" s="15"/>
       <c r="AD35" s="15"/>
-      <c r="AE35" s="15"/>
-      <c r="AF35" s="15"/>
-      <c r="AG35" s="15"/>
-      <c r="AH35" s="15"/>
+      <c r="AE35" s="16"/>
+      <c r="AF35" s="16"/>
+      <c r="AG35" s="16"/>
+      <c r="AH35" s="16"/>
       <c r="AI35" s="15"/>
       <c r="AJ35" s="15"/>
       <c r="AK35" s="15"/>
       <c r="AL35" s="15"/>
       <c r="AM35" s="15"/>
       <c r="AN35" s="15"/>
-      <c r="AO35" s="28"/>
+      <c r="AO35" s="15"/>
       <c r="AP35" s="15"/>
       <c r="AQ35" s="15"/>
       <c r="AR35" s="15"/>
-    </row>
-    <row r="36" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS35" s="15"/>
+      <c r="AT35" s="15"/>
+      <c r="AU35" s="28"/>
+      <c r="AV35" s="15"/>
+      <c r="AW35" s="15"/>
+      <c r="AX35" s="15"/>
+    </row>
+    <row r="36" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A36" s="17"/>
       <c r="B36" s="15"/>
       <c r="C36" s="15"/>
@@ -16694,22 +16914,28 @@
       <c r="AB36" s="15"/>
       <c r="AC36" s="15"/>
       <c r="AD36" s="15"/>
-      <c r="AE36" s="15"/>
-      <c r="AF36" s="15"/>
-      <c r="AG36" s="15"/>
-      <c r="AH36" s="15"/>
+      <c r="AE36" s="16"/>
+      <c r="AF36" s="16"/>
+      <c r="AG36" s="16"/>
+      <c r="AH36" s="16"/>
       <c r="AI36" s="15"/>
       <c r="AJ36" s="15"/>
       <c r="AK36" s="15"/>
       <c r="AL36" s="15"/>
       <c r="AM36" s="15"/>
       <c r="AN36" s="15"/>
-      <c r="AO36" s="28"/>
+      <c r="AO36" s="15"/>
       <c r="AP36" s="15"/>
       <c r="AQ36" s="15"/>
       <c r="AR36" s="15"/>
-    </row>
-    <row r="37" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS36" s="15"/>
+      <c r="AT36" s="15"/>
+      <c r="AU36" s="28"/>
+      <c r="AV36" s="15"/>
+      <c r="AW36" s="15"/>
+      <c r="AX36" s="15"/>
+    </row>
+    <row r="37" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A37" s="17"/>
       <c r="B37" s="15"/>
       <c r="C37" s="15"/>
@@ -16740,22 +16966,28 @@
       <c r="AB37" s="15"/>
       <c r="AC37" s="15"/>
       <c r="AD37" s="15"/>
-      <c r="AE37" s="15"/>
-      <c r="AF37" s="15"/>
-      <c r="AG37" s="15"/>
-      <c r="AH37" s="15"/>
+      <c r="AE37" s="16"/>
+      <c r="AF37" s="16"/>
+      <c r="AG37" s="16"/>
+      <c r="AH37" s="16"/>
       <c r="AI37" s="15"/>
       <c r="AJ37" s="15"/>
       <c r="AK37" s="15"/>
       <c r="AL37" s="15"/>
       <c r="AM37" s="15"/>
       <c r="AN37" s="15"/>
-      <c r="AO37" s="28"/>
+      <c r="AO37" s="15"/>
       <c r="AP37" s="15"/>
       <c r="AQ37" s="15"/>
       <c r="AR37" s="15"/>
-    </row>
-    <row r="38" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS37" s="15"/>
+      <c r="AT37" s="15"/>
+      <c r="AU37" s="28"/>
+      <c r="AV37" s="15"/>
+      <c r="AW37" s="15"/>
+      <c r="AX37" s="15"/>
+    </row>
+    <row r="38" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A38" s="17"/>
       <c r="B38" s="15"/>
       <c r="C38" s="15"/>
@@ -16786,22 +17018,28 @@
       <c r="AB38" s="15"/>
       <c r="AC38" s="15"/>
       <c r="AD38" s="15"/>
-      <c r="AE38" s="15"/>
-      <c r="AF38" s="15"/>
-      <c r="AG38" s="15"/>
-      <c r="AH38" s="15"/>
+      <c r="AE38" s="16"/>
+      <c r="AF38" s="16"/>
+      <c r="AG38" s="16"/>
+      <c r="AH38" s="16"/>
       <c r="AI38" s="15"/>
       <c r="AJ38" s="15"/>
       <c r="AK38" s="15"/>
       <c r="AL38" s="15"/>
       <c r="AM38" s="15"/>
       <c r="AN38" s="15"/>
-      <c r="AO38" s="28"/>
+      <c r="AO38" s="15"/>
       <c r="AP38" s="15"/>
       <c r="AQ38" s="15"/>
       <c r="AR38" s="15"/>
-    </row>
-    <row r="39" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS38" s="15"/>
+      <c r="AT38" s="15"/>
+      <c r="AU38" s="28"/>
+      <c r="AV38" s="15"/>
+      <c r="AW38" s="15"/>
+      <c r="AX38" s="15"/>
+    </row>
+    <row r="39" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A39" s="17"/>
       <c r="B39" s="15"/>
       <c r="C39" s="15"/>
@@ -16832,22 +17070,28 @@
       <c r="AB39" s="15"/>
       <c r="AC39" s="15"/>
       <c r="AD39" s="15"/>
-      <c r="AE39" s="15"/>
-      <c r="AF39" s="15"/>
-      <c r="AG39" s="15"/>
-      <c r="AH39" s="15"/>
+      <c r="AE39" s="16"/>
+      <c r="AF39" s="16"/>
+      <c r="AG39" s="16"/>
+      <c r="AH39" s="16"/>
       <c r="AI39" s="15"/>
       <c r="AJ39" s="15"/>
       <c r="AK39" s="15"/>
       <c r="AL39" s="15"/>
       <c r="AM39" s="15"/>
       <c r="AN39" s="15"/>
-      <c r="AO39" s="28"/>
+      <c r="AO39" s="15"/>
       <c r="AP39" s="15"/>
       <c r="AQ39" s="15"/>
       <c r="AR39" s="15"/>
-    </row>
-    <row r="40" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS39" s="15"/>
+      <c r="AT39" s="15"/>
+      <c r="AU39" s="28"/>
+      <c r="AV39" s="15"/>
+      <c r="AW39" s="15"/>
+      <c r="AX39" s="15"/>
+    </row>
+    <row r="40" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A40" s="17"/>
       <c r="B40" s="15"/>
       <c r="C40" s="15"/>
@@ -16878,22 +17122,28 @@
       <c r="AB40" s="15"/>
       <c r="AC40" s="15"/>
       <c r="AD40" s="15"/>
-      <c r="AE40" s="15"/>
-      <c r="AF40" s="15"/>
-      <c r="AG40" s="15"/>
-      <c r="AH40" s="15"/>
+      <c r="AE40" s="16"/>
+      <c r="AF40" s="16"/>
+      <c r="AG40" s="16"/>
+      <c r="AH40" s="16"/>
       <c r="AI40" s="15"/>
       <c r="AJ40" s="15"/>
       <c r="AK40" s="15"/>
       <c r="AL40" s="15"/>
       <c r="AM40" s="15"/>
       <c r="AN40" s="15"/>
-      <c r="AO40" s="28"/>
+      <c r="AO40" s="15"/>
       <c r="AP40" s="15"/>
       <c r="AQ40" s="15"/>
       <c r="AR40" s="15"/>
-    </row>
-    <row r="41" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS40" s="15"/>
+      <c r="AT40" s="15"/>
+      <c r="AU40" s="28"/>
+      <c r="AV40" s="15"/>
+      <c r="AW40" s="15"/>
+      <c r="AX40" s="15"/>
+    </row>
+    <row r="41" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A41" s="17"/>
       <c r="B41" s="15"/>
       <c r="C41" s="15"/>
@@ -16924,22 +17174,28 @@
       <c r="AB41" s="15"/>
       <c r="AC41" s="15"/>
       <c r="AD41" s="15"/>
-      <c r="AE41" s="15"/>
-      <c r="AF41" s="15"/>
-      <c r="AG41" s="15"/>
-      <c r="AH41" s="15"/>
+      <c r="AE41" s="16"/>
+      <c r="AF41" s="16"/>
+      <c r="AG41" s="16"/>
+      <c r="AH41" s="16"/>
       <c r="AI41" s="15"/>
       <c r="AJ41" s="15"/>
       <c r="AK41" s="15"/>
       <c r="AL41" s="15"/>
       <c r="AM41" s="15"/>
       <c r="AN41" s="15"/>
-      <c r="AO41" s="28"/>
+      <c r="AO41" s="15"/>
       <c r="AP41" s="15"/>
       <c r="AQ41" s="15"/>
       <c r="AR41" s="15"/>
-    </row>
-    <row r="42" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS41" s="15"/>
+      <c r="AT41" s="15"/>
+      <c r="AU41" s="28"/>
+      <c r="AV41" s="15"/>
+      <c r="AW41" s="15"/>
+      <c r="AX41" s="15"/>
+    </row>
+    <row r="42" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A42" s="17"/>
       <c r="B42" s="15"/>
       <c r="C42" s="15"/>
@@ -16970,22 +17226,28 @@
       <c r="AB42" s="15"/>
       <c r="AC42" s="15"/>
       <c r="AD42" s="15"/>
-      <c r="AE42" s="15"/>
-      <c r="AF42" s="15"/>
-      <c r="AG42" s="15"/>
-      <c r="AH42" s="15"/>
+      <c r="AE42" s="16"/>
+      <c r="AF42" s="16"/>
+      <c r="AG42" s="16"/>
+      <c r="AH42" s="16"/>
       <c r="AI42" s="15"/>
       <c r="AJ42" s="15"/>
       <c r="AK42" s="15"/>
       <c r="AL42" s="15"/>
       <c r="AM42" s="15"/>
       <c r="AN42" s="15"/>
-      <c r="AO42" s="28"/>
+      <c r="AO42" s="15"/>
       <c r="AP42" s="15"/>
       <c r="AQ42" s="15"/>
       <c r="AR42" s="15"/>
-    </row>
-    <row r="43" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS42" s="15"/>
+      <c r="AT42" s="15"/>
+      <c r="AU42" s="28"/>
+      <c r="AV42" s="15"/>
+      <c r="AW42" s="15"/>
+      <c r="AX42" s="15"/>
+    </row>
+    <row r="43" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A43" s="17"/>
       <c r="B43" s="15"/>
       <c r="C43" s="15"/>
@@ -17016,22 +17278,28 @@
       <c r="AB43" s="15"/>
       <c r="AC43" s="15"/>
       <c r="AD43" s="15"/>
-      <c r="AE43" s="15"/>
-      <c r="AF43" s="15"/>
-      <c r="AG43" s="15"/>
-      <c r="AH43" s="15"/>
+      <c r="AE43" s="16"/>
+      <c r="AF43" s="16"/>
+      <c r="AG43" s="16"/>
+      <c r="AH43" s="16"/>
       <c r="AI43" s="15"/>
       <c r="AJ43" s="15"/>
       <c r="AK43" s="15"/>
       <c r="AL43" s="15"/>
       <c r="AM43" s="15"/>
       <c r="AN43" s="15"/>
-      <c r="AO43" s="28"/>
+      <c r="AO43" s="15"/>
       <c r="AP43" s="15"/>
       <c r="AQ43" s="15"/>
       <c r="AR43" s="15"/>
-    </row>
-    <row r="44" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS43" s="15"/>
+      <c r="AT43" s="15"/>
+      <c r="AU43" s="28"/>
+      <c r="AV43" s="15"/>
+      <c r="AW43" s="15"/>
+      <c r="AX43" s="15"/>
+    </row>
+    <row r="44" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A44" s="17"/>
       <c r="B44" s="15"/>
       <c r="C44" s="15"/>
@@ -17062,22 +17330,28 @@
       <c r="AB44" s="15"/>
       <c r="AC44" s="15"/>
       <c r="AD44" s="15"/>
-      <c r="AE44" s="15"/>
-      <c r="AF44" s="15"/>
-      <c r="AG44" s="15"/>
-      <c r="AH44" s="15"/>
+      <c r="AE44" s="16"/>
+      <c r="AF44" s="16"/>
+      <c r="AG44" s="16"/>
+      <c r="AH44" s="16"/>
       <c r="AI44" s="15"/>
       <c r="AJ44" s="15"/>
       <c r="AK44" s="15"/>
       <c r="AL44" s="15"/>
       <c r="AM44" s="15"/>
       <c r="AN44" s="15"/>
-      <c r="AO44" s="28"/>
+      <c r="AO44" s="15"/>
       <c r="AP44" s="15"/>
       <c r="AQ44" s="15"/>
       <c r="AR44" s="15"/>
-    </row>
-    <row r="45" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS44" s="15"/>
+      <c r="AT44" s="15"/>
+      <c r="AU44" s="28"/>
+      <c r="AV44" s="15"/>
+      <c r="AW44" s="15"/>
+      <c r="AX44" s="15"/>
+    </row>
+    <row r="45" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A45" s="17"/>
       <c r="B45" s="15"/>
       <c r="C45" s="15"/>
@@ -17108,22 +17382,28 @@
       <c r="AB45" s="15"/>
       <c r="AC45" s="15"/>
       <c r="AD45" s="15"/>
-      <c r="AE45" s="15"/>
-      <c r="AF45" s="15"/>
-      <c r="AG45" s="15"/>
-      <c r="AH45" s="15"/>
+      <c r="AE45" s="16"/>
+      <c r="AF45" s="16"/>
+      <c r="AG45" s="16"/>
+      <c r="AH45" s="16"/>
       <c r="AI45" s="15"/>
       <c r="AJ45" s="15"/>
       <c r="AK45" s="15"/>
       <c r="AL45" s="15"/>
       <c r="AM45" s="15"/>
       <c r="AN45" s="15"/>
-      <c r="AO45" s="28"/>
+      <c r="AO45" s="15"/>
       <c r="AP45" s="15"/>
       <c r="AQ45" s="15"/>
       <c r="AR45" s="15"/>
-    </row>
-    <row r="46" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS45" s="15"/>
+      <c r="AT45" s="15"/>
+      <c r="AU45" s="28"/>
+      <c r="AV45" s="15"/>
+      <c r="AW45" s="15"/>
+      <c r="AX45" s="15"/>
+    </row>
+    <row r="46" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A46" s="17"/>
       <c r="B46" s="15"/>
       <c r="C46" s="15"/>
@@ -17154,22 +17434,28 @@
       <c r="AB46" s="15"/>
       <c r="AC46" s="15"/>
       <c r="AD46" s="15"/>
-      <c r="AE46" s="15"/>
-      <c r="AF46" s="15"/>
-      <c r="AG46" s="15"/>
-      <c r="AH46" s="15"/>
+      <c r="AE46" s="16"/>
+      <c r="AF46" s="16"/>
+      <c r="AG46" s="16"/>
+      <c r="AH46" s="16"/>
       <c r="AI46" s="15"/>
       <c r="AJ46" s="15"/>
       <c r="AK46" s="15"/>
       <c r="AL46" s="15"/>
       <c r="AM46" s="15"/>
       <c r="AN46" s="15"/>
-      <c r="AO46" s="28"/>
+      <c r="AO46" s="15"/>
       <c r="AP46" s="15"/>
       <c r="AQ46" s="15"/>
       <c r="AR46" s="15"/>
-    </row>
-    <row r="47" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS46" s="15"/>
+      <c r="AT46" s="15"/>
+      <c r="AU46" s="28"/>
+      <c r="AV46" s="15"/>
+      <c r="AW46" s="15"/>
+      <c r="AX46" s="15"/>
+    </row>
+    <row r="47" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A47" s="17"/>
       <c r="B47" s="15"/>
       <c r="C47" s="15"/>
@@ -17200,22 +17486,28 @@
       <c r="AB47" s="15"/>
       <c r="AC47" s="15"/>
       <c r="AD47" s="15"/>
-      <c r="AE47" s="15"/>
-      <c r="AF47" s="15"/>
-      <c r="AG47" s="15"/>
-      <c r="AH47" s="15"/>
+      <c r="AE47" s="16"/>
+      <c r="AF47" s="16"/>
+      <c r="AG47" s="16"/>
+      <c r="AH47" s="16"/>
       <c r="AI47" s="15"/>
       <c r="AJ47" s="15"/>
       <c r="AK47" s="15"/>
       <c r="AL47" s="15"/>
       <c r="AM47" s="15"/>
       <c r="AN47" s="15"/>
-      <c r="AO47" s="28"/>
+      <c r="AO47" s="15"/>
       <c r="AP47" s="15"/>
       <c r="AQ47" s="15"/>
       <c r="AR47" s="15"/>
-    </row>
-    <row r="48" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS47" s="15"/>
+      <c r="AT47" s="15"/>
+      <c r="AU47" s="28"/>
+      <c r="AV47" s="15"/>
+      <c r="AW47" s="15"/>
+      <c r="AX47" s="15"/>
+    </row>
+    <row r="48" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A48" s="17"/>
       <c r="B48" s="15"/>
       <c r="C48" s="15"/>
@@ -17246,22 +17538,28 @@
       <c r="AB48" s="15"/>
       <c r="AC48" s="15"/>
       <c r="AD48" s="15"/>
-      <c r="AE48" s="15"/>
-      <c r="AF48" s="15"/>
-      <c r="AG48" s="15"/>
-      <c r="AH48" s="15"/>
+      <c r="AE48" s="16"/>
+      <c r="AF48" s="16"/>
+      <c r="AG48" s="16"/>
+      <c r="AH48" s="16"/>
       <c r="AI48" s="15"/>
       <c r="AJ48" s="15"/>
       <c r="AK48" s="15"/>
       <c r="AL48" s="15"/>
       <c r="AM48" s="15"/>
       <c r="AN48" s="15"/>
-      <c r="AO48" s="28"/>
+      <c r="AO48" s="15"/>
       <c r="AP48" s="15"/>
       <c r="AQ48" s="15"/>
       <c r="AR48" s="15"/>
-    </row>
-    <row r="49" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS48" s="15"/>
+      <c r="AT48" s="15"/>
+      <c r="AU48" s="28"/>
+      <c r="AV48" s="15"/>
+      <c r="AW48" s="15"/>
+      <c r="AX48" s="15"/>
+    </row>
+    <row r="49" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A49" s="17"/>
       <c r="B49" s="15"/>
       <c r="C49" s="15"/>
@@ -17292,22 +17590,28 @@
       <c r="AB49" s="15"/>
       <c r="AC49" s="15"/>
       <c r="AD49" s="15"/>
-      <c r="AE49" s="15"/>
-      <c r="AF49" s="15"/>
-      <c r="AG49" s="15"/>
-      <c r="AH49" s="15"/>
+      <c r="AE49" s="16"/>
+      <c r="AF49" s="16"/>
+      <c r="AG49" s="16"/>
+      <c r="AH49" s="16"/>
       <c r="AI49" s="15"/>
       <c r="AJ49" s="15"/>
       <c r="AK49" s="15"/>
       <c r="AL49" s="15"/>
       <c r="AM49" s="15"/>
       <c r="AN49" s="15"/>
-      <c r="AO49" s="28"/>
+      <c r="AO49" s="15"/>
       <c r="AP49" s="15"/>
       <c r="AQ49" s="15"/>
       <c r="AR49" s="15"/>
-    </row>
-    <row r="50" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS49" s="15"/>
+      <c r="AT49" s="15"/>
+      <c r="AU49" s="28"/>
+      <c r="AV49" s="15"/>
+      <c r="AW49" s="15"/>
+      <c r="AX49" s="15"/>
+    </row>
+    <row r="50" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A50" s="17"/>
       <c r="B50" s="15"/>
       <c r="C50" s="15"/>
@@ -17338,22 +17642,28 @@
       <c r="AB50" s="15"/>
       <c r="AC50" s="15"/>
       <c r="AD50" s="15"/>
-      <c r="AE50" s="15"/>
-      <c r="AF50" s="15"/>
-      <c r="AG50" s="15"/>
-      <c r="AH50" s="15"/>
+      <c r="AE50" s="16"/>
+      <c r="AF50" s="16"/>
+      <c r="AG50" s="16"/>
+      <c r="AH50" s="16"/>
       <c r="AI50" s="15"/>
       <c r="AJ50" s="15"/>
       <c r="AK50" s="15"/>
       <c r="AL50" s="15"/>
       <c r="AM50" s="15"/>
       <c r="AN50" s="15"/>
-      <c r="AO50" s="28"/>
+      <c r="AO50" s="15"/>
       <c r="AP50" s="15"/>
       <c r="AQ50" s="15"/>
       <c r="AR50" s="15"/>
-    </row>
-    <row r="51" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS50" s="15"/>
+      <c r="AT50" s="15"/>
+      <c r="AU50" s="28"/>
+      <c r="AV50" s="15"/>
+      <c r="AW50" s="15"/>
+      <c r="AX50" s="15"/>
+    </row>
+    <row r="51" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A51" s="17"/>
       <c r="B51" s="15"/>
       <c r="C51" s="15"/>
@@ -17384,22 +17694,28 @@
       <c r="AB51" s="15"/>
       <c r="AC51" s="15"/>
       <c r="AD51" s="15"/>
-      <c r="AE51" s="15"/>
-      <c r="AF51" s="15"/>
-      <c r="AG51" s="15"/>
-      <c r="AH51" s="15"/>
+      <c r="AE51" s="16"/>
+      <c r="AF51" s="16"/>
+      <c r="AG51" s="16"/>
+      <c r="AH51" s="16"/>
       <c r="AI51" s="15"/>
       <c r="AJ51" s="15"/>
       <c r="AK51" s="15"/>
       <c r="AL51" s="15"/>
       <c r="AM51" s="15"/>
       <c r="AN51" s="15"/>
-      <c r="AO51" s="28"/>
+      <c r="AO51" s="15"/>
       <c r="AP51" s="15"/>
       <c r="AQ51" s="15"/>
       <c r="AR51" s="15"/>
-    </row>
-    <row r="52" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS51" s="15"/>
+      <c r="AT51" s="15"/>
+      <c r="AU51" s="28"/>
+      <c r="AV51" s="15"/>
+      <c r="AW51" s="15"/>
+      <c r="AX51" s="15"/>
+    </row>
+    <row r="52" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A52" s="17"/>
       <c r="B52" s="15"/>
       <c r="C52" s="15"/>
@@ -17430,20 +17746,26 @@
       <c r="AB52" s="15"/>
       <c r="AC52" s="15"/>
       <c r="AD52" s="15"/>
-      <c r="AE52" s="15"/>
-      <c r="AF52" s="15"/>
-      <c r="AG52" s="15"/>
-      <c r="AH52" s="15"/>
+      <c r="AE52" s="16"/>
+      <c r="AF52" s="16"/>
+      <c r="AG52" s="16"/>
+      <c r="AH52" s="16"/>
       <c r="AI52" s="15"/>
       <c r="AJ52" s="15"/>
       <c r="AK52" s="15"/>
       <c r="AL52" s="15"/>
       <c r="AM52" s="15"/>
       <c r="AN52" s="15"/>
-      <c r="AO52" s="28"/>
+      <c r="AO52" s="15"/>
       <c r="AP52" s="15"/>
       <c r="AQ52" s="15"/>
       <c r="AR52" s="15"/>
+      <c r="AS52" s="15"/>
+      <c r="AT52" s="15"/>
+      <c r="AU52" s="28"/>
+      <c r="AV52" s="15"/>
+      <c r="AW52" s="15"/>
+      <c r="AX52" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -17458,14 +17780,14 @@
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="B10:E10"/>
   </mergeCells>
-  <dataValidations count="14">
+  <dataValidations count="17">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Unique" prompt="A value must be unique within the dataset" sqref="H17:H52" xr:uid="{274C493E-CBE0-2742-BFD6-A161E5736B5A}">
       <formula1>"true,false"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C17:C52" xr:uid="{792BC06D-75E6-1A4B-8EE7-26D8A0C4CF46}">
       <formula1>"string,number,integer,boolean,array,object,timestamp,date,time,map,vector"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" sqref="B17:B52 J17:L52 O17:W52 Y17:AR52" xr:uid="{DDC4FF9F-5023-E04B-9FAD-8E0C431863DF}"/>
+    <dataValidation allowBlank="1" sqref="B17:B52 J17:L52 O17:W52 AR17:AX52 Y17:AM52" xr:uid="{DDC4FF9F-5023-E04B-9FAD-8E0C431863DF}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Required" prompt="Is this a required field (true) or can it be optional (false)" sqref="G17:G52" xr:uid="{653181B6-028C-9348-B6A1-78F7EF7B9A52}">
       <formula1>"true,false"</formula1>
     </dataValidation>
@@ -17481,15 +17803,24 @@
     <dataValidation type="list" allowBlank="1" sqref="X17:X52" xr:uid="{17C32F0F-20AB-664B-ABCA-B45524F93539}">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Comments" prompt="Use this for internal comments, open questions, discussion points. _x000a_This will not become part of the ODCS YAML." sqref="AO16" xr:uid="{D669647A-617C-7549-9EA2-AC37BFEA6E41}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Comments" prompt="Use this for internal comments, open questions, discussion points. _x000a_This will not become part of the ODCS YAML." sqref="AU16" xr:uid="{D669647A-617C-7549-9EA2-AC37BFEA6E41}"/>
     <dataValidation type="list" allowBlank="1" sqref="K17:K103" xr:uid="{FC6EF137-EF73-574C-95CF-B57336C59E8E}">
       <formula1>"column,measure,dimension"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="L17:L103" xr:uid="{A061E7B4-4C11-5241-BD09-1677165B8299}">
+    <dataValidation type="list" allowBlank="1" sqref="L17:L103 AQ17:AQ100" xr:uid="{A061E7B4-4C11-5241-BD09-1677165B8299}">
       <formula1>"true,false"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B14:E14" xr:uid="{D05E7DD6-9150-B941-B705-FF6CFA22D7F9}">
       <formula1>"true,false"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="AO17:AO100" xr:uid="{95DD2EA0-6986-414F-8048-0D9B55450EB2}">
+      <formula1>"bfloat16,binary,float16,float32,float64,int8,uint8"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="AP17:AP100" xr:uid="{EF98B3E8-396D-0F48-A972-E0956219870A}">
+      <formula1>"cosine,dotProduct,euclidean,hamming,manhattan"</formula1>
+    </dataValidation>
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" sqref="AN17:AN100" xr:uid="{F44F2772-48BF-B94D-9469-EC67E27A68CF}">
+      <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Excel: read the timezone, team tag and contract-created cells
</commit_message>
<xml_diff>
--- a/datacontract/templates/excel/odcs-template.xlsx
+++ b/datacontract/templates/excel/odcs-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jakob/entropyData/open-data-contract-standard-excel-template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB75899B-EBE7-F043-8A3F-9BE4C8EF552B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3875D753-AACC-B04A-B375-AAA28B30B143}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="-33240" windowWidth="60160" windowHeight="33240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="8" r:id="rId1"/>
@@ -39,20 +39,21 @@
     <definedName name="apiVersion">Fundamentals!$C$5</definedName>
     <definedName name="authoritativeDefinitions">'Authoritative Definitions'!$A$4:$F$1000</definedName>
     <definedName name="constraints">Constraints!$A$4:$AZ$1000</definedName>
-    <definedName name="context.instructions">Fundamentals!$C$25</definedName>
+    <definedName name="context.instructions">Fundamentals!$C$26</definedName>
+    <definedName name="contractCreatedTs">Fundamentals!$C$11</definedName>
     <definedName name="CustomProperties">'Custom Properties'!$A$5:$H$21</definedName>
     <definedName name="datacontract_id">Fundamentals!$C$7</definedName>
-    <definedName name="dataProduct">Fundamentals!$C$15</definedName>
-    <definedName name="description.limitations">Fundamentals!$C$20</definedName>
-    <definedName name="description.purpose">Fundamentals!$C$19</definedName>
-    <definedName name="description.usage">Fundamentals!$C$21</definedName>
-    <definedName name="domain">Fundamentals!$C$14</definedName>
+    <definedName name="dataProduct">Fundamentals!$C$16</definedName>
+    <definedName name="description.limitations">Fundamentals!$C$21</definedName>
+    <definedName name="description.purpose">Fundamentals!$C$20</definedName>
+    <definedName name="description.usage">Fundamentals!$C$22</definedName>
+    <definedName name="domain">Fundamentals!$C$15</definedName>
     <definedName name="enum">Enums!$A$4:$AZ$1000</definedName>
     <definedName name="id">Fundamentals!$C$7</definedName>
     <definedName name="instructions.importUrl">Instructions!$B$24</definedName>
     <definedName name="kind">Fundamentals!$C$4</definedName>
     <definedName name="name">Fundamentals!$C$8</definedName>
-    <definedName name="owner">Fundamentals!$C$12</definedName>
+    <definedName name="owner">Fundamentals!$C$13</definedName>
     <definedName name="price.id">Pricing!$B$7</definedName>
     <definedName name="price.priceAmount">Pricing!$B$4</definedName>
     <definedName name="price.priceCurrency">Pricing!$B$5</definedName>
@@ -69,7 +70,7 @@
     <definedName name="schema.name" localSheetId="2">'Schema &lt;table_name&gt;'!$B$5</definedName>
     <definedName name="schema.physicalName" localSheetId="2">'Schema &lt;table_name&gt;'!$B$9</definedName>
     <definedName name="schema.physicalType" localSheetId="2">'Schema &lt;table_name&gt;'!$B$6</definedName>
-    <definedName name="schema.properties" localSheetId="2">'Schema &lt;table_name&gt;'!$A$16:$AU$984</definedName>
+    <definedName name="schema.properties" localSheetId="2">'Schema &lt;table_name&gt;'!$A$16:$AW$984</definedName>
     <definedName name="schema.tags" localSheetId="2">'Schema &lt;table_name&gt;'!$B$11</definedName>
     <definedName name="servers.account">Servers!$C$11</definedName>
     <definedName name="servers.catalog">Servers!$C$12</definedName>
@@ -104,13 +105,13 @@
     <definedName name="status">Fundamentals!$C$10</definedName>
     <definedName name="support">Support!$A$4:$AZ$1000</definedName>
     <definedName name="synonyms">Synonyms!$A$4:$AZ$1000</definedName>
-    <definedName name="tags">Fundamentals!$C$23</definedName>
-    <definedName name="team">Team!$A$10:$AZ$1006</definedName>
+    <definedName name="tags">Fundamentals!$C$24</definedName>
+    <definedName name="team">Team!$A$10:$BA$1006</definedName>
     <definedName name="team.description">Team!$B$5</definedName>
     <definedName name="team.id">Team!$B$7</definedName>
     <definedName name="team.name">Team!$B$4</definedName>
     <definedName name="team.tags">Team!$B$6</definedName>
-    <definedName name="tenant">Fundamentals!$C$16</definedName>
+    <definedName name="tenant">Fundamentals!$C$17</definedName>
     <definedName name="verifiedStatements">'Verified Statements'!$A$4:$AZ$1000</definedName>
     <definedName name="version">Fundamentals!$C$9</definedName>
   </definedNames>
@@ -132,7 +133,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="260">
   <si>
     <t>Property</t>
   </si>
@@ -929,6 +930,15 @@
   </si>
   <si>
     <t>Text</t>
+  </si>
+  <si>
+    <t>Contract Created</t>
+  </si>
+  <si>
+    <t>Timezone</t>
+  </si>
+  <si>
+    <t>Default Timezone</t>
   </si>
 </sst>
 </file>
@@ -1148,7 +1158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1232,6 +1242,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -15392,7 +15405,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92ABE851-FB8B-2145-B7F8-5CF6722D55A6}">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.83203125" style="2" customWidth="1"/>
@@ -15470,32 +15483,31 @@
       <c r="C10" s="5"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="7"/>
+      <c r="A11" s="7" t="s">
+        <v>257</v>
+      </c>
       <c r="B11" s="7"/>
+      <c r="C11" s="34"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" s="34" t="s">
+      <c r="A12" s="7"/>
+      <c r="B12" s="7"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="35" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="35"/>
-      <c r="C12" s="5"/>
-      <c r="E12" s="6"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7"/>
+      <c r="B13" s="36"/>
+      <c r="C13" s="5"/>
+      <c r="E13" s="6"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="A14" s="7"/>
       <c r="B14" s="7"/>
-      <c r="C14" s="5"/>
-      <c r="E14" s="6"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="5"/>
@@ -15503,77 +15515,85 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B16" s="7"/>
       <c r="C16" s="5"/>
+      <c r="E16" s="6"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" s="7"/>
+      <c r="A17" s="7" t="s">
+        <v>27</v>
+      </c>
       <c r="B17" s="7"/>
+      <c r="C17" s="5"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="7"/>
+      <c r="B18" s="7"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B18" s="7"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" s="7"/>
-      <c r="B19" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="C19" s="5"/>
+      <c r="B19" s="7"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="7"/>
       <c r="B20" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C20" s="5"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="7"/>
       <c r="B21" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C21" s="5"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="7"/>
-      <c r="B22" s="7"/>
+      <c r="B22" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C22" s="5"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" s="7" t="s">
+      <c r="A23" s="7"/>
+      <c r="B23" s="7"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B23" s="7"/>
-      <c r="C23" s="5"/>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" s="7" t="s">
+      <c r="B24" s="7"/>
+      <c r="C24" s="5"/>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" s="7" t="s">
         <v>240</v>
       </c>
-      <c r="C25" s="5"/>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B26" s="2" t="s">
+      <c r="C26" s="5"/>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B27" s="2" t="s">
         <v>241</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" sqref="G11:L13 G17:L24" xr:uid="{7EB39568-B879-514E-B51D-6C44C6D6A95F}">
+    <dataValidation type="list" allowBlank="1" sqref="G12:L14 G18:L25" xr:uid="{7EB39568-B879-514E-B51D-6C44C6D6A95F}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="D22 D17:D18 D11:D13 D24" xr:uid="{1D2456BD-0546-F940-A9EF-51615EED43D0}">
+    <dataValidation type="list" allowBlank="1" sqref="D23 D18:D19 D12:D14 D25" xr:uid="{1D2456BD-0546-F940-A9EF-51615EED43D0}">
       <formula1>"string,number,integer,boolean,array,object"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Owner" prompt="The ID of the team owning the Data Contract._x000a_Required for Data Mesh Manager." sqref="C12" xr:uid="{35986E89-F1AF-D84C-96AD-8E5AC4A64A86}"/>
-    <dataValidation allowBlank="1" sqref="C11:C13 C17:C18 C22:C65" xr:uid="{D875F021-2666-244F-B1D7-40151775E3CC}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Owner" prompt="The ID of the team owning the Data Contract._x000a_Required for Data Mesh Manager." sqref="C13" xr:uid="{35986E89-F1AF-D84C-96AD-8E5AC4A64A86}"/>
+    <dataValidation allowBlank="1" sqref="C12:C14 C18:C19 C23:C66" xr:uid="{D875F021-2666-244F-B1D7-40151775E3CC}"/>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -15582,7 +15602,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AX52"/>
+  <dimension ref="A1:AZ52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.83203125" style="2" customWidth="1"/>
@@ -15603,122 +15623,122 @@
     <col min="18" max="22" width="19" style="2" customWidth="1"/>
     <col min="23" max="23" width="21.6640625" style="2" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="27.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="25" max="46" width="15.5" style="2" customWidth="1"/>
-    <col min="47" max="47" width="44.33203125" style="2" customWidth="1"/>
-    <col min="48" max="50" width="15.83203125" style="2" customWidth="1"/>
-    <col min="51" max="16384" width="8.83203125" style="2"/>
+    <col min="25" max="48" width="15.5" style="2" customWidth="1"/>
+    <col min="49" max="49" width="44.33203125" style="2" customWidth="1"/>
+    <col min="50" max="52" width="15.83203125" style="2" customWidth="1"/>
+    <col min="53" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:50" ht="24" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:52" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:50" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:50" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="5" spans="1:50" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="36" t="s">
+      <c r="B5" s="37" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="36"/>
-      <c r="D5" s="36"/>
-      <c r="E5" s="36"/>
-    </row>
-    <row r="6" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="C5" s="37"/>
+      <c r="D5" s="37"/>
+      <c r="E5" s="37"/>
+    </row>
+    <row r="6" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="37" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="36"/>
-      <c r="D6" s="36"/>
-      <c r="E6" s="36"/>
-    </row>
-    <row r="7" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="C6" s="37"/>
+      <c r="D6" s="37"/>
+      <c r="E6" s="37"/>
+    </row>
+    <row r="7" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="36"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
-    </row>
-    <row r="8" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="B7" s="37"/>
+      <c r="C7" s="37"/>
+      <c r="D7" s="37"/>
+      <c r="E7" s="37"/>
+    </row>
+    <row r="8" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="37"/>
-      <c r="C8" s="38"/>
-      <c r="D8" s="38"/>
-      <c r="E8" s="39"/>
-    </row>
-    <row r="9" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="B8" s="38"/>
+      <c r="C8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="40"/>
+    </row>
+    <row r="9" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B9" s="37"/>
-      <c r="C9" s="38"/>
-      <c r="D9" s="38"/>
-      <c r="E9" s="39"/>
-    </row>
-    <row r="10" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="B9" s="38"/>
+      <c r="C9" s="39"/>
+      <c r="D9" s="39"/>
+      <c r="E9" s="40"/>
+    </row>
+    <row r="10" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B10" s="37"/>
-      <c r="C10" s="38"/>
-      <c r="D10" s="38"/>
-      <c r="E10" s="39"/>
-    </row>
-    <row r="11" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="B10" s="38"/>
+      <c r="C10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="40"/>
+    </row>
+    <row r="11" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="36"/>
-      <c r="C11" s="36"/>
-      <c r="D11" s="36"/>
-      <c r="E11" s="36"/>
-    </row>
-    <row r="12" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="B11" s="37"/>
+      <c r="C11" s="37"/>
+      <c r="D11" s="37"/>
+      <c r="E11" s="37"/>
+    </row>
+    <row r="12" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="36"/>
-      <c r="C12" s="36"/>
-      <c r="D12" s="36"/>
-      <c r="E12" s="36"/>
-    </row>
-    <row r="13" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="B12" s="37"/>
+      <c r="C12" s="37"/>
+      <c r="D12" s="37"/>
+      <c r="E12" s="37"/>
+    </row>
+    <row r="13" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="B13" s="36"/>
-      <c r="C13" s="36"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="36"/>
-    </row>
-    <row r="14" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="B13" s="37"/>
+      <c r="C13" s="37"/>
+      <c r="D13" s="37"/>
+      <c r="E13" s="37"/>
+    </row>
+    <row r="14" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
         <v>218</v>
       </c>
-      <c r="B14" s="36"/>
-      <c r="C14" s="36"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="36"/>
-    </row>
-    <row r="15" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="B14" s="37"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="37"/>
+      <c r="E14" s="37"/>
+    </row>
+    <row r="15" spans="1:52" x14ac:dyDescent="0.2">
       <c r="E15" s="2"/>
       <c r="Y15" s="19" t="s">
         <v>77</v>
@@ -15742,14 +15762,16 @@
       <c r="AP15" s="20"/>
       <c r="AQ15" s="20"/>
       <c r="AR15" s="20"/>
-      <c r="AS15" s="21"/>
-      <c r="AV15" s="19" t="s">
+      <c r="AS15" s="20"/>
+      <c r="AT15" s="20"/>
+      <c r="AU15" s="21"/>
+      <c r="AX15" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="AW15" s="20"/>
-      <c r="AX15" s="20"/>
-    </row>
-    <row r="16" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY15" s="20"/>
+      <c r="AZ15" s="20"/>
+    </row>
+    <row r="16" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
         <v>0</v>
       </c>
@@ -15886,16 +15908,22 @@
         <v>254</v>
       </c>
       <c r="AT16" s="10" t="s">
+        <v>258</v>
+      </c>
+      <c r="AU16" s="10" t="s">
+        <v>259</v>
+      </c>
+      <c r="AV16" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="AU16" s="10" t="s">
+      <c r="AW16" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="AV16" s="10"/>
-      <c r="AW16" s="10"/>
       <c r="AX16" s="10"/>
-    </row>
-    <row r="17" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY16" s="10"/>
+      <c r="AZ16" s="10"/>
+    </row>
+    <row r="17" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A17" s="17"/>
       <c r="B17" s="15"/>
       <c r="C17" s="15"/>
@@ -15942,12 +15970,14 @@
       <c r="AR17" s="15"/>
       <c r="AS17" s="15"/>
       <c r="AT17" s="15"/>
-      <c r="AU17" s="28"/>
+      <c r="AU17" s="15"/>
       <c r="AV17" s="15"/>
-      <c r="AW17" s="15"/>
+      <c r="AW17" s="28"/>
       <c r="AX17" s="15"/>
-    </row>
-    <row r="18" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY17" s="15"/>
+      <c r="AZ17" s="15"/>
+    </row>
+    <row r="18" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A18" s="17"/>
       <c r="B18" s="15"/>
       <c r="C18" s="15"/>
@@ -15994,12 +16024,14 @@
       <c r="AR18" s="15"/>
       <c r="AS18" s="15"/>
       <c r="AT18" s="15"/>
-      <c r="AU18" s="28"/>
+      <c r="AU18" s="15"/>
       <c r="AV18" s="15"/>
-      <c r="AW18" s="15"/>
+      <c r="AW18" s="28"/>
       <c r="AX18" s="15"/>
-    </row>
-    <row r="19" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY18" s="15"/>
+      <c r="AZ18" s="15"/>
+    </row>
+    <row r="19" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A19" s="17"/>
       <c r="B19" s="15"/>
       <c r="C19" s="15"/>
@@ -16046,12 +16078,14 @@
       <c r="AR19" s="15"/>
       <c r="AS19" s="15"/>
       <c r="AT19" s="15"/>
-      <c r="AU19" s="28"/>
+      <c r="AU19" s="15"/>
       <c r="AV19" s="15"/>
-      <c r="AW19" s="15"/>
+      <c r="AW19" s="28"/>
       <c r="AX19" s="15"/>
-    </row>
-    <row r="20" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY19" s="15"/>
+      <c r="AZ19" s="15"/>
+    </row>
+    <row r="20" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A20" s="17"/>
       <c r="B20" s="15"/>
       <c r="C20" s="15"/>
@@ -16098,12 +16132,14 @@
       <c r="AR20" s="15"/>
       <c r="AS20" s="15"/>
       <c r="AT20" s="15"/>
-      <c r="AU20" s="28"/>
+      <c r="AU20" s="15"/>
       <c r="AV20" s="15"/>
-      <c r="AW20" s="15"/>
+      <c r="AW20" s="28"/>
       <c r="AX20" s="15"/>
-    </row>
-    <row r="21" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY20" s="15"/>
+      <c r="AZ20" s="15"/>
+    </row>
+    <row r="21" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A21" s="17"/>
       <c r="B21" s="15"/>
       <c r="C21" s="15"/>
@@ -16150,12 +16186,14 @@
       <c r="AR21" s="15"/>
       <c r="AS21" s="15"/>
       <c r="AT21" s="15"/>
-      <c r="AU21" s="28"/>
+      <c r="AU21" s="15"/>
       <c r="AV21" s="15"/>
-      <c r="AW21" s="15"/>
+      <c r="AW21" s="28"/>
       <c r="AX21" s="15"/>
-    </row>
-    <row r="22" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY21" s="15"/>
+      <c r="AZ21" s="15"/>
+    </row>
+    <row r="22" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A22" s="17"/>
       <c r="B22" s="15"/>
       <c r="C22" s="15"/>
@@ -16202,12 +16240,14 @@
       <c r="AR22" s="15"/>
       <c r="AS22" s="15"/>
       <c r="AT22" s="15"/>
-      <c r="AU22" s="28"/>
+      <c r="AU22" s="15"/>
       <c r="AV22" s="15"/>
-      <c r="AW22" s="15"/>
+      <c r="AW22" s="28"/>
       <c r="AX22" s="15"/>
-    </row>
-    <row r="23" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY22" s="15"/>
+      <c r="AZ22" s="15"/>
+    </row>
+    <row r="23" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A23" s="17"/>
       <c r="B23" s="15"/>
       <c r="C23" s="15"/>
@@ -16254,12 +16294,14 @@
       <c r="AR23" s="15"/>
       <c r="AS23" s="15"/>
       <c r="AT23" s="15"/>
-      <c r="AU23" s="28"/>
+      <c r="AU23" s="15"/>
       <c r="AV23" s="15"/>
-      <c r="AW23" s="15"/>
+      <c r="AW23" s="28"/>
       <c r="AX23" s="15"/>
-    </row>
-    <row r="24" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY23" s="15"/>
+      <c r="AZ23" s="15"/>
+    </row>
+    <row r="24" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A24" s="18"/>
       <c r="B24" s="15"/>
       <c r="C24" s="15"/>
@@ -16306,12 +16348,14 @@
       <c r="AR24" s="15"/>
       <c r="AS24" s="15"/>
       <c r="AT24" s="15"/>
-      <c r="AU24" s="28"/>
+      <c r="AU24" s="15"/>
       <c r="AV24" s="15"/>
-      <c r="AW24" s="15"/>
+      <c r="AW24" s="28"/>
       <c r="AX24" s="15"/>
-    </row>
-    <row r="25" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY24" s="15"/>
+      <c r="AZ24" s="15"/>
+    </row>
+    <row r="25" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A25" s="18"/>
       <c r="B25" s="15"/>
       <c r="C25" s="15"/>
@@ -16358,12 +16402,14 @@
       <c r="AR25" s="15"/>
       <c r="AS25" s="15"/>
       <c r="AT25" s="15"/>
-      <c r="AU25" s="28"/>
+      <c r="AU25" s="15"/>
       <c r="AV25" s="15"/>
-      <c r="AW25" s="15"/>
+      <c r="AW25" s="28"/>
       <c r="AX25" s="15"/>
-    </row>
-    <row r="26" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY25" s="15"/>
+      <c r="AZ25" s="15"/>
+    </row>
+    <row r="26" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A26" s="18"/>
       <c r="B26" s="15"/>
       <c r="C26" s="15"/>
@@ -16410,12 +16456,14 @@
       <c r="AR26" s="15"/>
       <c r="AS26" s="15"/>
       <c r="AT26" s="15"/>
-      <c r="AU26" s="28"/>
+      <c r="AU26" s="15"/>
       <c r="AV26" s="15"/>
-      <c r="AW26" s="15"/>
+      <c r="AW26" s="28"/>
       <c r="AX26" s="15"/>
-    </row>
-    <row r="27" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY26" s="15"/>
+      <c r="AZ26" s="15"/>
+    </row>
+    <row r="27" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A27" s="17"/>
       <c r="B27" s="15"/>
       <c r="C27" s="15"/>
@@ -16462,12 +16510,14 @@
       <c r="AR27" s="15"/>
       <c r="AS27" s="15"/>
       <c r="AT27" s="15"/>
-      <c r="AU27" s="28"/>
+      <c r="AU27" s="15"/>
       <c r="AV27" s="15"/>
-      <c r="AW27" s="15"/>
+      <c r="AW27" s="28"/>
       <c r="AX27" s="15"/>
-    </row>
-    <row r="28" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY27" s="15"/>
+      <c r="AZ27" s="15"/>
+    </row>
+    <row r="28" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A28" s="17"/>
       <c r="B28" s="15"/>
       <c r="C28" s="15"/>
@@ -16514,12 +16564,14 @@
       <c r="AR28" s="15"/>
       <c r="AS28" s="15"/>
       <c r="AT28" s="15"/>
-      <c r="AU28" s="28"/>
+      <c r="AU28" s="15"/>
       <c r="AV28" s="15"/>
-      <c r="AW28" s="15"/>
+      <c r="AW28" s="28"/>
       <c r="AX28" s="15"/>
-    </row>
-    <row r="29" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY28" s="15"/>
+      <c r="AZ28" s="15"/>
+    </row>
+    <row r="29" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A29" s="17"/>
       <c r="B29" s="15"/>
       <c r="C29" s="15"/>
@@ -16566,12 +16618,14 @@
       <c r="AR29" s="15"/>
       <c r="AS29" s="15"/>
       <c r="AT29" s="15"/>
-      <c r="AU29" s="28"/>
+      <c r="AU29" s="15"/>
       <c r="AV29" s="15"/>
-      <c r="AW29" s="15"/>
+      <c r="AW29" s="28"/>
       <c r="AX29" s="15"/>
-    </row>
-    <row r="30" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY29" s="15"/>
+      <c r="AZ29" s="15"/>
+    </row>
+    <row r="30" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A30" s="17"/>
       <c r="B30" s="15"/>
       <c r="C30" s="15"/>
@@ -16618,12 +16672,14 @@
       <c r="AR30" s="15"/>
       <c r="AS30" s="15"/>
       <c r="AT30" s="15"/>
-      <c r="AU30" s="28"/>
+      <c r="AU30" s="15"/>
       <c r="AV30" s="15"/>
-      <c r="AW30" s="15"/>
+      <c r="AW30" s="28"/>
       <c r="AX30" s="15"/>
-    </row>
-    <row r="31" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY30" s="15"/>
+      <c r="AZ30" s="15"/>
+    </row>
+    <row r="31" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A31" s="17"/>
       <c r="B31" s="15"/>
       <c r="C31" s="15"/>
@@ -16670,12 +16726,14 @@
       <c r="AR31" s="15"/>
       <c r="AS31" s="15"/>
       <c r="AT31" s="15"/>
-      <c r="AU31" s="28"/>
+      <c r="AU31" s="15"/>
       <c r="AV31" s="15"/>
-      <c r="AW31" s="15"/>
+      <c r="AW31" s="28"/>
       <c r="AX31" s="15"/>
-    </row>
-    <row r="32" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY31" s="15"/>
+      <c r="AZ31" s="15"/>
+    </row>
+    <row r="32" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A32" s="17"/>
       <c r="B32" s="15"/>
       <c r="C32" s="15"/>
@@ -16722,12 +16780,14 @@
       <c r="AR32" s="15"/>
       <c r="AS32" s="15"/>
       <c r="AT32" s="15"/>
-      <c r="AU32" s="28"/>
+      <c r="AU32" s="15"/>
       <c r="AV32" s="15"/>
-      <c r="AW32" s="15"/>
+      <c r="AW32" s="28"/>
       <c r="AX32" s="15"/>
-    </row>
-    <row r="33" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY32" s="15"/>
+      <c r="AZ32" s="15"/>
+    </row>
+    <row r="33" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A33" s="17"/>
       <c r="B33" s="15"/>
       <c r="C33" s="15"/>
@@ -16774,12 +16834,14 @@
       <c r="AR33" s="15"/>
       <c r="AS33" s="15"/>
       <c r="AT33" s="15"/>
-      <c r="AU33" s="28"/>
+      <c r="AU33" s="15"/>
       <c r="AV33" s="15"/>
-      <c r="AW33" s="15"/>
+      <c r="AW33" s="28"/>
       <c r="AX33" s="15"/>
-    </row>
-    <row r="34" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY33" s="15"/>
+      <c r="AZ33" s="15"/>
+    </row>
+    <row r="34" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A34" s="17"/>
       <c r="B34" s="15"/>
       <c r="C34" s="15"/>
@@ -16826,12 +16888,14 @@
       <c r="AR34" s="15"/>
       <c r="AS34" s="15"/>
       <c r="AT34" s="15"/>
-      <c r="AU34" s="28"/>
+      <c r="AU34" s="15"/>
       <c r="AV34" s="15"/>
-      <c r="AW34" s="15"/>
+      <c r="AW34" s="28"/>
       <c r="AX34" s="15"/>
-    </row>
-    <row r="35" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY34" s="15"/>
+      <c r="AZ34" s="15"/>
+    </row>
+    <row r="35" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A35" s="17"/>
       <c r="B35" s="15"/>
       <c r="C35" s="15"/>
@@ -16878,12 +16942,14 @@
       <c r="AR35" s="15"/>
       <c r="AS35" s="15"/>
       <c r="AT35" s="15"/>
-      <c r="AU35" s="28"/>
+      <c r="AU35" s="15"/>
       <c r="AV35" s="15"/>
-      <c r="AW35" s="15"/>
+      <c r="AW35" s="28"/>
       <c r="AX35" s="15"/>
-    </row>
-    <row r="36" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY35" s="15"/>
+      <c r="AZ35" s="15"/>
+    </row>
+    <row r="36" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A36" s="17"/>
       <c r="B36" s="15"/>
       <c r="C36" s="15"/>
@@ -16930,12 +16996,14 @@
       <c r="AR36" s="15"/>
       <c r="AS36" s="15"/>
       <c r="AT36" s="15"/>
-      <c r="AU36" s="28"/>
+      <c r="AU36" s="15"/>
       <c r="AV36" s="15"/>
-      <c r="AW36" s="15"/>
+      <c r="AW36" s="28"/>
       <c r="AX36" s="15"/>
-    </row>
-    <row r="37" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY36" s="15"/>
+      <c r="AZ36" s="15"/>
+    </row>
+    <row r="37" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A37" s="17"/>
       <c r="B37" s="15"/>
       <c r="C37" s="15"/>
@@ -16982,12 +17050,14 @@
       <c r="AR37" s="15"/>
       <c r="AS37" s="15"/>
       <c r="AT37" s="15"/>
-      <c r="AU37" s="28"/>
+      <c r="AU37" s="15"/>
       <c r="AV37" s="15"/>
-      <c r="AW37" s="15"/>
+      <c r="AW37" s="28"/>
       <c r="AX37" s="15"/>
-    </row>
-    <row r="38" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY37" s="15"/>
+      <c r="AZ37" s="15"/>
+    </row>
+    <row r="38" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A38" s="17"/>
       <c r="B38" s="15"/>
       <c r="C38" s="15"/>
@@ -17034,12 +17104,14 @@
       <c r="AR38" s="15"/>
       <c r="AS38" s="15"/>
       <c r="AT38" s="15"/>
-      <c r="AU38" s="28"/>
+      <c r="AU38" s="15"/>
       <c r="AV38" s="15"/>
-      <c r="AW38" s="15"/>
+      <c r="AW38" s="28"/>
       <c r="AX38" s="15"/>
-    </row>
-    <row r="39" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY38" s="15"/>
+      <c r="AZ38" s="15"/>
+    </row>
+    <row r="39" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A39" s="17"/>
       <c r="B39" s="15"/>
       <c r="C39" s="15"/>
@@ -17086,12 +17158,14 @@
       <c r="AR39" s="15"/>
       <c r="AS39" s="15"/>
       <c r="AT39" s="15"/>
-      <c r="AU39" s="28"/>
+      <c r="AU39" s="15"/>
       <c r="AV39" s="15"/>
-      <c r="AW39" s="15"/>
+      <c r="AW39" s="28"/>
       <c r="AX39" s="15"/>
-    </row>
-    <row r="40" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY39" s="15"/>
+      <c r="AZ39" s="15"/>
+    </row>
+    <row r="40" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A40" s="17"/>
       <c r="B40" s="15"/>
       <c r="C40" s="15"/>
@@ -17138,12 +17212,14 @@
       <c r="AR40" s="15"/>
       <c r="AS40" s="15"/>
       <c r="AT40" s="15"/>
-      <c r="AU40" s="28"/>
+      <c r="AU40" s="15"/>
       <c r="AV40" s="15"/>
-      <c r="AW40" s="15"/>
+      <c r="AW40" s="28"/>
       <c r="AX40" s="15"/>
-    </row>
-    <row r="41" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY40" s="15"/>
+      <c r="AZ40" s="15"/>
+    </row>
+    <row r="41" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A41" s="17"/>
       <c r="B41" s="15"/>
       <c r="C41" s="15"/>
@@ -17190,12 +17266,14 @@
       <c r="AR41" s="15"/>
       <c r="AS41" s="15"/>
       <c r="AT41" s="15"/>
-      <c r="AU41" s="28"/>
+      <c r="AU41" s="15"/>
       <c r="AV41" s="15"/>
-      <c r="AW41" s="15"/>
+      <c r="AW41" s="28"/>
       <c r="AX41" s="15"/>
-    </row>
-    <row r="42" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY41" s="15"/>
+      <c r="AZ41" s="15"/>
+    </row>
+    <row r="42" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A42" s="17"/>
       <c r="B42" s="15"/>
       <c r="C42" s="15"/>
@@ -17242,12 +17320,14 @@
       <c r="AR42" s="15"/>
       <c r="AS42" s="15"/>
       <c r="AT42" s="15"/>
-      <c r="AU42" s="28"/>
+      <c r="AU42" s="15"/>
       <c r="AV42" s="15"/>
-      <c r="AW42" s="15"/>
+      <c r="AW42" s="28"/>
       <c r="AX42" s="15"/>
-    </row>
-    <row r="43" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY42" s="15"/>
+      <c r="AZ42" s="15"/>
+    </row>
+    <row r="43" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A43" s="17"/>
       <c r="B43" s="15"/>
       <c r="C43" s="15"/>
@@ -17294,12 +17374,14 @@
       <c r="AR43" s="15"/>
       <c r="AS43" s="15"/>
       <c r="AT43" s="15"/>
-      <c r="AU43" s="28"/>
+      <c r="AU43" s="15"/>
       <c r="AV43" s="15"/>
-      <c r="AW43" s="15"/>
+      <c r="AW43" s="28"/>
       <c r="AX43" s="15"/>
-    </row>
-    <row r="44" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY43" s="15"/>
+      <c r="AZ43" s="15"/>
+    </row>
+    <row r="44" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A44" s="17"/>
       <c r="B44" s="15"/>
       <c r="C44" s="15"/>
@@ -17346,12 +17428,14 @@
       <c r="AR44" s="15"/>
       <c r="AS44" s="15"/>
       <c r="AT44" s="15"/>
-      <c r="AU44" s="28"/>
+      <c r="AU44" s="15"/>
       <c r="AV44" s="15"/>
-      <c r="AW44" s="15"/>
+      <c r="AW44" s="28"/>
       <c r="AX44" s="15"/>
-    </row>
-    <row r="45" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY44" s="15"/>
+      <c r="AZ44" s="15"/>
+    </row>
+    <row r="45" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A45" s="17"/>
       <c r="B45" s="15"/>
       <c r="C45" s="15"/>
@@ -17398,12 +17482,14 @@
       <c r="AR45" s="15"/>
       <c r="AS45" s="15"/>
       <c r="AT45" s="15"/>
-      <c r="AU45" s="28"/>
+      <c r="AU45" s="15"/>
       <c r="AV45" s="15"/>
-      <c r="AW45" s="15"/>
+      <c r="AW45" s="28"/>
       <c r="AX45" s="15"/>
-    </row>
-    <row r="46" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY45" s="15"/>
+      <c r="AZ45" s="15"/>
+    </row>
+    <row r="46" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A46" s="17"/>
       <c r="B46" s="15"/>
       <c r="C46" s="15"/>
@@ -17450,12 +17536,14 @@
       <c r="AR46" s="15"/>
       <c r="AS46" s="15"/>
       <c r="AT46" s="15"/>
-      <c r="AU46" s="28"/>
+      <c r="AU46" s="15"/>
       <c r="AV46" s="15"/>
-      <c r="AW46" s="15"/>
+      <c r="AW46" s="28"/>
       <c r="AX46" s="15"/>
-    </row>
-    <row r="47" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY46" s="15"/>
+      <c r="AZ46" s="15"/>
+    </row>
+    <row r="47" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A47" s="17"/>
       <c r="B47" s="15"/>
       <c r="C47" s="15"/>
@@ -17502,12 +17590,14 @@
       <c r="AR47" s="15"/>
       <c r="AS47" s="15"/>
       <c r="AT47" s="15"/>
-      <c r="AU47" s="28"/>
+      <c r="AU47" s="15"/>
       <c r="AV47" s="15"/>
-      <c r="AW47" s="15"/>
+      <c r="AW47" s="28"/>
       <c r="AX47" s="15"/>
-    </row>
-    <row r="48" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY47" s="15"/>
+      <c r="AZ47" s="15"/>
+    </row>
+    <row r="48" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A48" s="17"/>
       <c r="B48" s="15"/>
       <c r="C48" s="15"/>
@@ -17554,12 +17644,14 @@
       <c r="AR48" s="15"/>
       <c r="AS48" s="15"/>
       <c r="AT48" s="15"/>
-      <c r="AU48" s="28"/>
+      <c r="AU48" s="15"/>
       <c r="AV48" s="15"/>
-      <c r="AW48" s="15"/>
+      <c r="AW48" s="28"/>
       <c r="AX48" s="15"/>
-    </row>
-    <row r="49" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY48" s="15"/>
+      <c r="AZ48" s="15"/>
+    </row>
+    <row r="49" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A49" s="17"/>
       <c r="B49" s="15"/>
       <c r="C49" s="15"/>
@@ -17606,12 +17698,14 @@
       <c r="AR49" s="15"/>
       <c r="AS49" s="15"/>
       <c r="AT49" s="15"/>
-      <c r="AU49" s="28"/>
+      <c r="AU49" s="15"/>
       <c r="AV49" s="15"/>
-      <c r="AW49" s="15"/>
+      <c r="AW49" s="28"/>
       <c r="AX49" s="15"/>
-    </row>
-    <row r="50" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY49" s="15"/>
+      <c r="AZ49" s="15"/>
+    </row>
+    <row r="50" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A50" s="17"/>
       <c r="B50" s="15"/>
       <c r="C50" s="15"/>
@@ -17658,12 +17752,14 @@
       <c r="AR50" s="15"/>
       <c r="AS50" s="15"/>
       <c r="AT50" s="15"/>
-      <c r="AU50" s="28"/>
+      <c r="AU50" s="15"/>
       <c r="AV50" s="15"/>
-      <c r="AW50" s="15"/>
+      <c r="AW50" s="28"/>
       <c r="AX50" s="15"/>
-    </row>
-    <row r="51" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY50" s="15"/>
+      <c r="AZ50" s="15"/>
+    </row>
+    <row r="51" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A51" s="17"/>
       <c r="B51" s="15"/>
       <c r="C51" s="15"/>
@@ -17710,12 +17806,14 @@
       <c r="AR51" s="15"/>
       <c r="AS51" s="15"/>
       <c r="AT51" s="15"/>
-      <c r="AU51" s="28"/>
+      <c r="AU51" s="15"/>
       <c r="AV51" s="15"/>
-      <c r="AW51" s="15"/>
+      <c r="AW51" s="28"/>
       <c r="AX51" s="15"/>
-    </row>
-    <row r="52" spans="1:50" x14ac:dyDescent="0.2">
+      <c r="AY51" s="15"/>
+      <c r="AZ51" s="15"/>
+    </row>
+    <row r="52" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A52" s="17"/>
       <c r="B52" s="15"/>
       <c r="C52" s="15"/>
@@ -17762,10 +17860,12 @@
       <c r="AR52" s="15"/>
       <c r="AS52" s="15"/>
       <c r="AT52" s="15"/>
-      <c r="AU52" s="28"/>
+      <c r="AU52" s="15"/>
       <c r="AV52" s="15"/>
-      <c r="AW52" s="15"/>
+      <c r="AW52" s="28"/>
       <c r="AX52" s="15"/>
+      <c r="AY52" s="15"/>
+      <c r="AZ52" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -17787,7 +17887,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C17:C52" xr:uid="{792BC06D-75E6-1A4B-8EE7-26D8A0C4CF46}">
       <formula1>"string,number,integer,boolean,array,object,timestamp,date,time,map,vector"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" sqref="B17:B52 J17:L52 O17:W52 AR17:AX52 Y17:AM52" xr:uid="{DDC4FF9F-5023-E04B-9FAD-8E0C431863DF}"/>
+    <dataValidation allowBlank="1" sqref="B17:B52 J17:L52 O17:W52 Y17:AM52 AR17:AS52 AU17:AZ52" xr:uid="{DDC4FF9F-5023-E04B-9FAD-8E0C431863DF}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Required" prompt="Is this a required field (true) or can it be optional (false)" sqref="G17:G52" xr:uid="{653181B6-028C-9348-B6A1-78F7EF7B9A52}">
       <formula1>"true,false"</formula1>
     </dataValidation>
@@ -17803,11 +17903,11 @@
     <dataValidation type="list" allowBlank="1" sqref="X17:X52" xr:uid="{17C32F0F-20AB-664B-ABCA-B45524F93539}">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Comments" prompt="Use this for internal comments, open questions, discussion points. _x000a_This will not become part of the ODCS YAML." sqref="AU16" xr:uid="{D669647A-617C-7549-9EA2-AC37BFEA6E41}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Comments" prompt="Use this for internal comments, open questions, discussion points. _x000a_This will not become part of the ODCS YAML." sqref="AW16" xr:uid="{D669647A-617C-7549-9EA2-AC37BFEA6E41}"/>
     <dataValidation type="list" allowBlank="1" sqref="K17:K103" xr:uid="{FC6EF137-EF73-574C-95CF-B57336C59E8E}">
       <formula1>"column,measure,dimension"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="L17:L103 AQ17:AQ100" xr:uid="{A061E7B4-4C11-5241-BD09-1677165B8299}">
+    <dataValidation type="list" allowBlank="1" sqref="L17:L103 AQ17:AQ100 AT17:AT100" xr:uid="{A061E7B4-4C11-5241-BD09-1677165B8299}">
       <formula1>"true,false"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B14:E14" xr:uid="{D05E7DD6-9150-B941-B705-FF6CFA22D7F9}">
@@ -18971,65 +19071,65 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD55E6DF-E5C5-C142-BA93-791862A30BE7}">
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="33.1640625" style="2" customWidth="1"/>
     <col min="2" max="3" width="59.6640625" style="2" customWidth="1"/>
-    <col min="4" max="7" width="23.6640625" style="2" customWidth="1"/>
-    <col min="8" max="8" width="23.5" style="2" customWidth="1"/>
-    <col min="9" max="11" width="15.83203125" style="2" customWidth="1"/>
-    <col min="12" max="16384" width="8.83203125" style="2"/>
+    <col min="4" max="8" width="23.6640625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="23.5" style="2" customWidth="1"/>
+    <col min="10" max="12" width="15.83203125" style="2" customWidth="1"/>
+    <col min="13" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="4"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
         <v>156</v>
       </c>
       <c r="B4" s="5"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="5"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B6" s="5"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
         <v>22</v>
       </c>
       <c r="B7" s="5"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="4"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="I9" s="19" t="s">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="J9" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="J9" s="20"/>
       <c r="K9" s="20"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L9" s="20"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
         <v>62</v>
       </c>
@@ -19043,245 +19143,265 @@
         <v>63</v>
       </c>
       <c r="E10" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="G10" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="G10" s="10" t="s">
+      <c r="H10" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="I10" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="I10" s="10"/>
       <c r="J10" s="10"/>
       <c r="K10" s="10"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L10" s="10"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
+      <c r="F11" s="34"/>
+      <c r="G11" s="34"/>
       <c r="H11" s="5"/>
-      <c r="I11" s="15"/>
+      <c r="I11" s="5"/>
       <c r="J11" s="15"/>
       <c r="K11" s="15"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L11" s="15"/>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
+      <c r="F12" s="34"/>
+      <c r="G12" s="34"/>
       <c r="H12" s="5"/>
-      <c r="I12" s="15"/>
+      <c r="I12" s="5"/>
       <c r="J12" s="15"/>
       <c r="K12" s="15"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L12" s="15"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="34"/>
       <c r="H13" s="5"/>
-      <c r="I13" s="15"/>
+      <c r="I13" s="5"/>
       <c r="J13" s="15"/>
       <c r="K13" s="15"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L13" s="15"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
+      <c r="F14" s="34"/>
+      <c r="G14" s="34"/>
       <c r="H14" s="5"/>
-      <c r="I14" s="15"/>
+      <c r="I14" s="5"/>
       <c r="J14" s="15"/>
       <c r="K14" s="15"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L14" s="15"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
+      <c r="F15" s="34"/>
+      <c r="G15" s="34"/>
       <c r="H15" s="5"/>
-      <c r="I15" s="15"/>
+      <c r="I15" s="5"/>
       <c r="J15" s="15"/>
       <c r="K15" s="15"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L15" s="15"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
+      <c r="F16" s="34"/>
+      <c r="G16" s="34"/>
       <c r="H16" s="5"/>
-      <c r="I16" s="15"/>
+      <c r="I16" s="5"/>
       <c r="J16" s="15"/>
       <c r="K16" s="15"/>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L16" s="15"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
+      <c r="F17" s="34"/>
+      <c r="G17" s="34"/>
       <c r="H17" s="5"/>
-      <c r="I17" s="15"/>
+      <c r="I17" s="5"/>
       <c r="J17" s="15"/>
       <c r="K17" s="15"/>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L17" s="15"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
+      <c r="F18" s="34"/>
+      <c r="G18" s="34"/>
       <c r="H18" s="5"/>
-      <c r="I18" s="15"/>
+      <c r="I18" s="5"/>
       <c r="J18" s="15"/>
       <c r="K18" s="15"/>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L18" s="15"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="5"/>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
       <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
+      <c r="F19" s="34"/>
+      <c r="G19" s="34"/>
       <c r="H19" s="5"/>
-      <c r="I19" s="15"/>
+      <c r="I19" s="5"/>
       <c r="J19" s="15"/>
       <c r="K19" s="15"/>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L19" s="15"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
       <c r="D20" s="5"/>
       <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
+      <c r="F20" s="34"/>
+      <c r="G20" s="34"/>
       <c r="H20" s="5"/>
-      <c r="I20" s="15"/>
+      <c r="I20" s="5"/>
       <c r="J20" s="15"/>
       <c r="K20" s="15"/>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L20" s="15"/>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="5"/>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
       <c r="D21" s="5"/>
       <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
+      <c r="F21" s="34"/>
+      <c r="G21" s="34"/>
       <c r="H21" s="5"/>
-      <c r="I21" s="15"/>
+      <c r="I21" s="5"/>
       <c r="J21" s="15"/>
       <c r="K21" s="15"/>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L21" s="15"/>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="5"/>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
       <c r="D22" s="5"/>
       <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
+      <c r="F22" s="34"/>
+      <c r="G22" s="34"/>
       <c r="H22" s="5"/>
-      <c r="I22" s="15"/>
+      <c r="I22" s="5"/>
       <c r="J22" s="15"/>
       <c r="K22" s="15"/>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L22" s="15"/>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="5"/>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
       <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
+      <c r="F23" s="34"/>
+      <c r="G23" s="34"/>
       <c r="H23" s="5"/>
-      <c r="I23" s="15"/>
+      <c r="I23" s="5"/>
       <c r="J23" s="15"/>
       <c r="K23" s="15"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L23" s="15"/>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="5"/>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
       <c r="D24" s="5"/>
       <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
+      <c r="F24" s="34"/>
+      <c r="G24" s="34"/>
       <c r="H24" s="5"/>
-      <c r="I24" s="15"/>
+      <c r="I24" s="5"/>
       <c r="J24" s="15"/>
       <c r="K24" s="15"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L24" s="15"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="5"/>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
       <c r="D25" s="5"/>
       <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
-      <c r="G25" s="5"/>
+      <c r="F25" s="34"/>
+      <c r="G25" s="34"/>
       <c r="H25" s="5"/>
-      <c r="I25" s="15"/>
+      <c r="I25" s="5"/>
       <c r="J25" s="15"/>
       <c r="K25" s="15"/>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L25" s="15"/>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="5"/>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
       <c r="D26" s="5"/>
       <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
-      <c r="G26" s="5"/>
+      <c r="F26" s="34"/>
+      <c r="G26" s="34"/>
       <c r="H26" s="5"/>
-      <c r="I26" s="15"/>
+      <c r="I26" s="5"/>
       <c r="J26" s="15"/>
       <c r="K26" s="15"/>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L26" s="15"/>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="5"/>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
       <c r="E27" s="5"/>
-      <c r="F27" s="5"/>
-      <c r="G27" s="5"/>
+      <c r="F27" s="34"/>
+      <c r="G27" s="34"/>
       <c r="H27" s="5"/>
-      <c r="I27" s="15"/>
+      <c r="I27" s="5"/>
       <c r="J27" s="15"/>
       <c r="K27" s="15"/>
+      <c r="L27" s="15"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="1" sqref="B11:G67 H11:K27" xr:uid="{8BD676B5-0F0C-9D41-BB36-24C33963E434}"/>
+    <dataValidation allowBlank="1" sqref="B11:H67 I11:L27" xr:uid="{8BD676B5-0F0C-9D41-BB36-24C33963E434}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>